<commit_message>
Move pooled mandates out of fund vehicles
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -3315,17 +3315,17 @@
       </c>
       <c r="E35" s="23" t="inlineStr">
         <is>
-          <t>Include</t>
+          <t>Move to Pipeline &amp; Mandates</t>
         </is>
       </c>
       <c r="F35" s="23" t="inlineStr">
         <is>
-          <t>Include - aggregate actual pooled mandate</t>
+          <t>Moved - aggregate pooled mandate</t>
         </is>
       </c>
       <c r="G35" s="23" t="inlineStr">
         <is>
-          <t>Retain as aggregate consortium archetype, not as a conventional fund LP row. IFC reports KEPFIC mobilized $113m into two housing projects and facilitated two member-fund investments; MiDA reports Lot 3 Road Project Bonds investment by KEPFIC members.</t>
+          <t>Aggregate pooled mandate / consortium archetype, not a conventional fund vehicle LP row. Kept out of Fund Vehicles and Commitments Database to avoid treating a mandate platform as a fund commitment.</t>
         </is>
       </c>
       <c r="H35" s="23" t="inlineStr">
@@ -3539,17 +3539,17 @@
       </c>
       <c r="E41" s="23" t="inlineStr">
         <is>
-          <t>Include</t>
+          <t>Move to Pipeline &amp; Mandates</t>
         </is>
       </c>
       <c r="F41" s="23" t="inlineStr">
         <is>
-          <t>Include - aggregate actual pooled mandate</t>
+          <t>Moved - aggregate pooled mandate</t>
         </is>
       </c>
       <c r="G41" s="23" t="inlineStr">
         <is>
-          <t>Retain as aggregate consortium archetype. Engineering News reports AOFSA member funds collectively committed R5.7bn to infrastructure; MiDA/USAID sources also report &gt;$400m commitments.</t>
+          <t>Aggregate pooled mandate / consortium archetype, not a conventional fund vehicle LP row. Kept out of Fund Vehicles and Commitments Database to avoid treating a mandate platform as a fund commitment.</t>
         </is>
       </c>
       <c r="H41" s="23" t="inlineStr">
@@ -31365,7 +31365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="16" min="1" max="1"/>
@@ -32440,6 +32440,170 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>KEPFIC (Kenya Pension Funds Investment Consortium)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Pension consortium / pooled mandate</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Pooled mandate / aggregate evidence</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Various managers via KEPFIC consortium</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>KEPFIC pooled mandates (Kenya)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Infrastructure / Alts</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Kenya + regional</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2019-ongoing</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>USD 113m mobilized into two housing projects; member AUM ~USD 5bn</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Aggregate consortium / pooled mandate</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>IFC 2023; MiDA Advisors</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Aggregate pooled mandate / consortium archetype, not a conventional fund vehicle LP row. Kept out of Fund Vehicles and Commitments Database to avoid treating a mandate platform as a fund commitment.</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>https://www.ifc.org/en/stories/2023/pooling-pensions-in-kenya ; https://www.midaadvisors.com/advisory-firm-financing-the-development-of-critical-infrastructure-in-kenya-with-local-institutional-capital</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Asset Owners Forum of South Africa (AOFSA)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Pension consortium / pooled mandate</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Pooled mandate / aggregate evidence</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Various managers via AOFSA consortium</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>AOFSA pooled infrastructure mandates (South Africa)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Infrastructure / Alts</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2021-ongoing</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>R5.7bn / USD 400m+ collectively committed to infrastructure and other alternatives</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ZAR / USD</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Aggregate consortium / pooled mandate</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Engineering News 2022; MiDA/USAID AOFSA case materials</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Aggregate pooled mandate / consortium archetype, not a conventional fund vehicle LP row. Kept out of Fund Vehicles and Commitments Database to avoid treating a mandate platform as a fund commitment.</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>https://www.engineeringnews.co.za/article/aofsa-exceeds-infrastructure-investment-target-as-it-marks-first-anniversary-2022-11-21 ; https://www.midaadvisors.com/advisory-firm-what-we-do/institutional-investors-capacity-development</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:P13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -32452,7 +32616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="16" min="1" max="1"/>
@@ -33997,104 +34161,106 @@
     <row r="29" ht="45.75" customHeight="1" s="16">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>KEPFIC pooled mandates (Kenya)</t>
+          <t>Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN)</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Various (mandates allocated to managers)</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>2019-ongoing</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>USD 113m mobilized into two housing projects; member AUM ~USD 5bn</t>
-        </is>
+          <t>Sahel Capital</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>65.90000000000001</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Infrastructure / alts</t>
+          <t>PE / Agribusiness</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Kenya + regional</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>24 member schemes</t>
-        </is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>24 Kenyan retirement benefit funds (named on KEPFIC site); collective ~1/3 of total Kenyan pension AUM</t>
+          <t>NSIA Nigeria</t>
         </is>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
+          <t>AfDB, BII, Dutch Good Growth Fund</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>USAID + World Bank Group technical support; FMA Kenya MOU</t>
-        </is>
-      </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Aggregate consortium archetype, not a conventional fund LP row. Retained because IFC reports two facilitated member-fund investments and $113m mobilized; MiDA reports members invested in Lot 3 Road Project Bonds.</t>
+          <t>NSIA's earliest disclosed PE fund LP position; alongside three DFIs.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="90.75" customHeight="1" s="16">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN)</t>
+          <t>Capital Alliance Private Equity I-IV (CAPE)</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Sahel Capital</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>2017</v>
-      </c>
-      <c r="D30" s="2" t="n">
-        <v>65.90000000000001</v>
+          <t>African Capital Alliance (ACA)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>1998-ongoing</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>&gt;1,000 cumulative</t>
+        </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>PE / Agribusiness</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="n">
-        <v>1</v>
+          <t>Nigeria + West Africa</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>historical cohort</t>
+        </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>NSIA Nigeria</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="n">
-        <v>3</v>
+          <t>Nigerian PFAs (categorical historical disclosure; ACA explicitly 'championed PE inclusion as allowable Nigerian pension asset class')</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>multiple</t>
+        </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>AfDB, BII, Dutch Good Growth Fund</t>
+          <t>BII (CAPE IV); various DFIs across vintages</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -34104,59 +34270,53 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>NSIA's earliest disclosed PE fund LP position; alongside three DFIs.</t>
+          <t>First Nigerian PE firm (founded 1997); CAPE I was Nigeria's first PE fund (1998). Continental pioneer of pension-PE inclusion.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="23.25" customHeight="1" s="16">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Capital Alliance Private Equity I-IV (CAPE)</t>
+          <t>Rwanda SME Growth Fund</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>African Capital Alliance (ACA)</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>1998-ongoing</t>
-        </is>
+          <t>Enko Capital (Rwanda subsidiary)</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>2026</v>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>&gt;1,000 cumulative</t>
+          <t>30 first close (target 100)</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PE / SME growth (local-currency)</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Nigeria + West Africa</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>historical cohort</t>
-        </is>
+          <t>Rwanda</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Nigerian PFAs (categorical historical disclosure; ACA explicitly 'championed PE inclusion as allowable Nigerian pension asset class')</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>multiple</t>
-        </is>
+          <t>RSSB (Rwanda Social Security Board) — USD 30m anchor + USD 3m TA seed</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>BII (CAPE IV); various DFIs across vintages</t>
+          <t>FSD Africa Investments (structuring + planned guarantee)</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -34166,105 +34326,105 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>First Nigerian PE firm (founded 1997); CAPE I was Nigeria's first PE fund (1998). Continental pioneer of pension-PE inclusion.</t>
+          <t>First permanent capital vehicle anchored by an African pension fund (per RSSB CEO). Three regional firsts: pension-fund-led SME-only mandate, anchor permanent-capital vehicle, pension-fund TA facility.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="23.25" customHeight="1" s="16">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Rwanda SME Growth Fund</t>
+          <t>Mirepa Capital SME Fund I</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Enko Capital (Rwanda subsidiary)</t>
+          <t>Mirepa Investment Advisors</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>30 first close (target 100)</t>
+          <t>~10-12 (GHS 120m initial close)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>PE / SME growth (local-currency)</t>
+          <t>PE / SME growth</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Rwanda</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="n">
-        <v>1</v>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>2 named pension trustees + categorical CAMCOL schemes</t>
+        </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>RSSB (Rwanda Social Security Board) — USD 30m anchor + USD 3m TA seed</t>
+          <t>Petra Trust; Axis Pensions; multiple schemes via CAL Asset Management Company (CAMCOL); Venture Capital Trust Fund (VCTF)</t>
         </is>
       </c>
       <c r="I32" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>FSD Africa Investments (structuring + planned guarantee)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VCTF is a Ghanaian quasi-government VC fund (not strictly a DFI)</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>First permanent capital vehicle anchored by an African pension fund (per RSSB CEO). Three regional firsts: pension-fund-led SME-only mandate, anchor permanent-capital vehicle, pension-fund TA facility.</t>
+          <t>Second Ghana fund anchored solely by local investors (after Injaro IGVCF). 100% local-LP-funded. Confirms Ghana's emerging mandated-minimum-alts policy is producing real deal flow.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="23.25" customHeight="1" s="16">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>AOFSA pooled infrastructure mandates (South Africa)</t>
+          <t>Injaro Ghana Venture Capital Fund (IGVCF)</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Various managers (mandates allocated)</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>2021-ongoing</t>
-        </is>
+          <t>Injaro Investment Advisors</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>2023</v>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>R5.7bn / USD 400m+ collectively committed to infrastructure and other alternatives</t>
+          <t>~17.4 (GHS 216m final close Dec 2023)</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Infrastructure / Alts</t>
+          <t>PE / SME / VC</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Ghana + Côte d'Ivoire</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>12-15 member schemes</t>
+          <t>multiple Ghanaian pension funds (anchor cohort)</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>GEPF; EPPF; Telkom Retirement Fund; Transnet Retirement Fund; National Fund for Municipal Workers; KZN Joint Municipal Pension Fund (NJMPF); KZN Municipal Pension Fund; Motor Industry Retirement Fund (named); 4-7 additional founding members not individually named</t>
+          <t>Specific names not individually disclosed</t>
         </is>
       </c>
       <c r="I33" s="2" t="n">
@@ -34277,131 +34437,17 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Batseta Council; USAID + MiDA Advisors + World Bank technical support</t>
+          <t>Venture Capital Trust Fund (VCTF) of Ghana</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Aggregate consortium archetype, not a conventional fund LP row. Retained because public sources report actual collective member commitments, while individual member rows are not separately counted as commitments.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="23.25" customHeight="1" s="16">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Mirepa Capital SME Fund I</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Mirepa Investment Advisors</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>~10-12 (GHS 120m initial close)</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>PE / SME growth</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>2 named pension trustees + categorical CAMCOL schemes</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>Petra Trust; Axis Pensions; multiple schemes via CAL Asset Management Company (CAMCOL); Venture Capital Trust Fund (VCTF)</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>VCTF is a Ghanaian quasi-government VC fund (not strictly a DFI)</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>Second Ghana fund anchored solely by local investors (after Injaro IGVCF). 100% local-LP-funded. Confirms Ghana's emerging mandated-minimum-alts policy is producing real deal flow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="23.25" customHeight="1" s="16">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Injaro Ghana Venture Capital Fund (IGVCF)</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Injaro Investment Advisors</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>~17.4 (GHS 216m final close Dec 2023)</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>PE / SME / VC</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>Ghana + Côte d'Ivoire</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>multiple Ghanaian pension funds (anchor cohort)</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>Specific names not individually disclosed</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>Venture Capital Trust Fund (VCTF) of Ghana</t>
-        </is>
-      </c>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
           <t>FIRST Ghana fund of its kind anchored by local pension funds. Historical precedent for Mirepa I, Ci-Gaba, GIP Ghana model. Ghana cedi-denominated.</t>
         </is>
       </c>
     </row>
+    <row r="34" ht="23.25" customHeight="1" s="16"/>
+    <row r="35" ht="23.25" customHeight="1" s="16"/>
     <row r="36" ht="15" customHeight="1" s="16"/>
     <row r="37" ht="34.5" customHeight="1" s="16"/>
     <row r="38" ht="23.25" customHeight="1" s="16"/>
@@ -36911,7 +36957,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="15" customHeight="1" s="16">
       <c r="A19" s="18" t="inlineStr">
         <is>
@@ -36927,7 +36972,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Africa Food Security Fund
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -2035,7 +2035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="16" min="1" max="1"/>
@@ -4074,6 +4074,43 @@
       </c>
       <c r="H56" s="23" t="inlineStr"/>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Funds &amp; LP Co-Investors</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Africa Food Security Fund (AFSF)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>PIC on behalf of GEPF (South Africa)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Include - confirmed African PF/SWF LP</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>DGGF names PIC on behalf of GEPF as a first-round investor in AFSF alongside DFIs and DGGF; this is confirmed African pension fund involvement in a fund vehicle.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://english.dggf.nl/latest/news/2019/01/24/zebu-s-africa-food-security-fund-a-dggf-investee-reaches-total-fund-size-of-usd-84-million</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4086,7 +4123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F178"/>
+  <dimension ref="A1:F179"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="16" min="1" max="2"/>
@@ -9789,6 +9826,38 @@
       <c r="F178" s="2" t="inlineStr">
         <is>
           <t>Kenya Cabinet-approved National Infrastructure Fund + SWF; KPC IPO planned March 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>GEPF / PIC</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>DFI / fund announcement</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>DGGF - Zebu Africa Food Security Fund reaches total fund size of USD 84 million</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>https://english.dggf.nl/latest/news/2019/01/24/zebu-s-africa-food-security-fund-a-dggf-investee-reaches-total-fund-size-of-usd-84-million</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>PIC/GEPF LP confirmation in Africa Food Security Fund; co-investors AfDB, CDC/BII, DGGF, IFU, EBID and Kuramo</t>
         </is>
       </c>
     </row>
@@ -24770,7 +24839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O86"/>
+  <dimension ref="A1:O87"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="16" min="1" max="1"/>
@@ -31329,7 +31398,81 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="34.5" customHeight="1" s="16"/>
+    <row r="87" ht="34.5" customHeight="1" s="16">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>GEPF / PIC (South Africa)</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Public PF (via asset manager)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Zebu Investment Partners</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Africa Food Security Fund (AFSF)</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>PE / agriculture / food security</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>2019</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Not disclosed; fund size USD 84m</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>DFI / fund close announcement</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>DGGF news release, Jan 2019</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>DGGF names PIC on behalf of GEPF among first-round AFSF investors alongside AfDB, CDC Group/BII, DGGF, IFU, and EBID; Kuramo later joined, bringing fund commitments to USD 84m.</t>
+        </is>
+      </c>
+    </row>
     <row r="88" ht="45.75" customHeight="1" s="16"/>
     <row r="89" ht="34.5" customHeight="1" s="16"/>
     <row r="90" ht="34.5" customHeight="1" s="16"/>
@@ -32616,7 +32759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="16" min="1" max="1"/>
@@ -34446,7 +34589,60 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="23.25" customHeight="1" s="16"/>
+    <row r="34" ht="23.25" customHeight="1" s="16">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Africa Food Security Fund (AFSF)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Zebu Investment Partners</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D34" t="n">
+        <v>84</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>PE / agriculture / food security</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>PIC on behalf of GEPF (South Africa)</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>5</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>AfDB; BII (CDC Group); Dutch Good Growth Fund (DGGF); IFU; EBID</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Kuramo Capital Management</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>DGGF news release names PIC/GEPF in first-round investor group alongside DFIs and DGGF; Kuramo subsequently joined to bring commitments to USD 84m.</t>
+        </is>
+      </c>
+    </row>
     <row r="35" ht="23.25" customHeight="1" s="16"/>
     <row r="36" ht="15" customHeight="1" s="16"/>
     <row r="37" ht="34.5" customHeight="1" s="16"/>
@@ -34475,7 +34671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="16" min="1" max="1"/>
@@ -34526,11 +34722,11 @@
         </is>
       </c>
       <c r="B4" s="23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C4" s="23" t="inlineStr">
         <is>
-          <t>Ascent Rift Valley Fund II (ARVF II); Capital Alliance Private Equity I-IV (CAPE); Catalyst Fund II; Growth Investment Partners (GIP) Ghana; Growth Investment Partners (GIP) Zambia; Helios Investors II/III/IV (historical); Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Vantage Mezzanine IV (Pan-African sub-fund)</t>
+          <t>Ascent Rift Valley Fund II (ARVF II); Capital Alliance Private Equity I-IV (CAPE); Catalyst Fund II; Growth Investment Partners (GIP) Ghana; Growth Investment Partners (GIP) Zambia; Helios Investors II/III/IV (historical); Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Vantage Mezzanine IV (Pan-African sub-fund); Africa Food Security Fund (AFSF)</t>
         </is>
       </c>
       <c r="D4" s="23" t="inlineStr">
@@ -34551,11 +34747,11 @@
         </is>
       </c>
       <c r="B5" s="23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C5" s="23" t="inlineStr">
         <is>
-          <t>AfricInvest FIVE (Financial Inclusion Vehicle); Africa50 (general); Africa50 Infrastructure Acceleration Fund (IAF); Mediterrania Capital II / III / IV; Nigeria Infrastructure Fund (NIF, NSIA sub-fund); Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN)</t>
+          <t>AfricInvest FIVE (Financial Inclusion Vehicle); Africa50 (general); Africa50 Infrastructure Acceleration Fund (IAF); Mediterrania Capital II / III / IV; Nigeria Infrastructure Fund (NIF, NSIA sub-fund); Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Africa Food Security Fund (AFSF)</t>
         </is>
       </c>
       <c r="D5" s="23" t="inlineStr">
@@ -35026,11 +35222,11 @@
         </is>
       </c>
       <c r="B24" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN)</t>
+          <t>Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Africa Food Security Fund (AFSF)</t>
         </is>
       </c>
       <c r="D24" s="23" t="inlineStr">
@@ -35101,11 +35297,11 @@
         </is>
       </c>
       <c r="B27" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" s="23" t="inlineStr">
         <is>
-          <t>AfricInvest FIVE (Financial Inclusion Vehicle)</t>
+          <t>AfricInvest FIVE (Financial Inclusion Vehicle); Africa Food Security Fund (AFSF)</t>
         </is>
       </c>
       <c r="D27" s="23" t="inlineStr">
@@ -35236,6 +35432,56 @@
     <row r="46" ht="23.85" customHeight="1" s="16"/>
     <row r="47" ht="23.85" customHeight="1" s="16"/>
     <row r="48" ht="129.75" customHeight="1" s="16"/>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>EBID</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Africa Food Security Fund (AFSF)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>3 (Selective / TA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Kuramo Capital Management</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Africa Food Security Fund (AFSF)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Other named LP / fund-of-funds investor appearing in retained vehicles with African PF/SWF participation.</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>3 (Selective / TA)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:E27"/>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Add omission scan audit workflow
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -16,10 +16,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Country Summary" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology &amp; Caveats" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inclusion Audit" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Library" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Absentees Investigation" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regulatory vs Behaviour" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AVCA Aggregate vs Disclosed" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Omission Candidates" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Library" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Absentees Investigation" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regulatory vs Behaviour" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AVCA Aggregate vs Disclosed" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sovereign Wealth Funds'!$A$1:$K$27</definedName>
@@ -30,9 +31,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Funds &amp; LP Co-Investors'!$A$1:$L$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'DFI Co-Investor Patterns'!$A$3:$E$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Inclusion Audit'!$A$1:$H$56</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Source Library'!$A$1:$F$178</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Absentees Investigation'!$A$3:$G$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Regulatory vs Behaviour'!$A$3:$H$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Source Library'!$A$1:$F$178</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Absentees Investigation'!$A$3:$G$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Regulatory vs Behaviour'!$A$3:$H$22</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -103,7 +104,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -130,6 +131,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="007A4E00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A3A5C"/>
       </patternFill>
     </fill>
   </fills>
@@ -198,7 +204,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -264,6 +270,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4123,6 +4132,444 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:P5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" style="16" min="1" max="1"/>
+    <col width="34" customWidth="1" style="16" min="2" max="2"/>
+    <col width="24" customWidth="1" style="16" min="3" max="3"/>
+    <col width="34" customWidth="1" style="16" min="4" max="4"/>
+    <col width="38" customWidth="1" style="16" min="5" max="5"/>
+    <col width="20" customWidth="1" style="16" min="6" max="6"/>
+    <col width="20" customWidth="1" style="16" min="7" max="7"/>
+    <col width="14" customWidth="1" style="16" min="8" max="8"/>
+    <col width="34" customWidth="1" style="16" min="9" max="9"/>
+    <col width="12" customWidth="1" style="16" min="10" max="10"/>
+    <col width="42" customWidth="1" style="16" min="11" max="11"/>
+    <col width="52" customWidth="1" style="16" min="12" max="12"/>
+    <col width="58" customWidth="1" style="16" min="13" max="13"/>
+    <col width="58" customWidth="1" style="16" min="14" max="14"/>
+    <col width="24" customWidth="1" style="16" min="15" max="15"/>
+    <col width="14" customWidth="1" style="16" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>Candidate status</t>
+        </is>
+      </c>
+      <c r="B1" s="27" t="inlineStr">
+        <is>
+          <t>Vehicle</t>
+        </is>
+      </c>
+      <c r="C1" s="27" t="inlineStr">
+        <is>
+          <t>Manager / GP</t>
+        </is>
+      </c>
+      <c r="D1" s="27" t="inlineStr">
+        <is>
+          <t>African PF/SWF evidence</t>
+        </is>
+      </c>
+      <c r="E1" s="27" t="inlineStr">
+        <is>
+          <t>DFI / Other LP evidence</t>
+        </is>
+      </c>
+      <c r="F1" s="27" t="inlineStr">
+        <is>
+          <t>Asset class</t>
+        </is>
+      </c>
+      <c r="G1" s="27" t="inlineStr">
+        <is>
+          <t>Geographic focus</t>
+        </is>
+      </c>
+      <c r="H1" s="27" t="inlineStr">
+        <is>
+          <t>Vintage / year</t>
+        </is>
+      </c>
+      <c r="I1" s="27" t="inlineStr">
+        <is>
+          <t>Fund size / commitment evidence</t>
+        </is>
+      </c>
+      <c r="J1" s="27" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="K1" s="27" t="inlineStr">
+        <is>
+          <t>Recommended action</t>
+        </is>
+      </c>
+      <c r="L1" s="27" t="inlineStr">
+        <is>
+          <t>Evidence summary</t>
+        </is>
+      </c>
+      <c r="M1" s="27" t="inlineStr">
+        <is>
+          <t>Primary source URL</t>
+        </is>
+      </c>
+      <c r="N1" s="27" t="inlineStr">
+        <is>
+          <t>Secondary source URL</t>
+        </is>
+      </c>
+      <c r="O1" s="27" t="inlineStr">
+        <is>
+          <t>Search batch</t>
+        </is>
+      </c>
+      <c r="P1" s="27" t="inlineStr">
+        <is>
+          <t>Date added</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>Actioned - added to database</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>Africa Food Security Fund (AFSF)</t>
+        </is>
+      </c>
+      <c r="C2" s="21" t="inlineStr">
+        <is>
+          <t>Zebu Investment Partners</t>
+        </is>
+      </c>
+      <c r="D2" s="21" t="inlineStr">
+        <is>
+          <t>PIC on behalf of GEPF (South Africa)</t>
+        </is>
+      </c>
+      <c r="E2" s="21" t="inlineStr">
+        <is>
+          <t>AfDB; CDC Group/BII; Dutch Good Growth Fund; IFU; EBID; Kuramo Capital Management</t>
+        </is>
+      </c>
+      <c r="F2" s="21" t="inlineStr">
+        <is>
+          <t>PE / agriculture / food security</t>
+        </is>
+      </c>
+      <c r="G2" s="21" t="inlineStr">
+        <is>
+          <t>Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="H2" s="21" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="I2" s="21" t="inlineStr">
+        <is>
+          <t>DGGF says AFSF reached USD 84m; BII page says total commitments USD 90m</t>
+        </is>
+      </c>
+      <c r="J2" s="21" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="K2" s="21" t="inlineStr">
+        <is>
+          <t>Already added to Commitments, Fund Vehicles, Source Library, Inclusion Audit, and DFI/Other LP patterns.</t>
+        </is>
+      </c>
+      <c r="L2" s="21" t="inlineStr">
+        <is>
+          <t>DGGF names PIC on behalf of GEPF in first-round investors alongside DFIs and DGGF; BII confirms CDC invested alongside PIC and DFI group.</t>
+        </is>
+      </c>
+      <c r="M2" s="21" t="inlineStr">
+        <is>
+          <t>https://english.dggf.nl/latest/news/2019/01/24/zebu-s-africa-food-security-fund-a-dggf-investee-reaches-total-fund-size-of-usd-84-million</t>
+        </is>
+      </c>
+      <c r="N2" s="21" t="inlineStr">
+        <is>
+          <t>https://www.bii.co.uk/en/our-impact/fund/africa-food-security-fund-i-investment-01/</t>
+        </is>
+      </c>
+      <c r="O2" s="21" t="inlineStr">
+        <is>
+          <t>PIC/GEPF + DFI sweep</t>
+        </is>
+      </c>
+      <c r="P2" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="21" t="inlineStr">
+        <is>
+          <t>Candidate - likely add after row construction</t>
+        </is>
+      </c>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>Pan African Infrastructure Development Fund (PAIDF)</t>
+        </is>
+      </c>
+      <c r="C3" s="21" t="inlineStr">
+        <is>
+          <t>PAIDF Management Company / Harith-linked platform</t>
+        </is>
+      </c>
+      <c r="D3" s="21" t="inlineStr">
+        <is>
+          <t>PIC/GEPF; Eskom Pension and Provident Fund; SSNIT Ghana; Metropolitan/Old Mutual/Stanlib named in source context</t>
+        </is>
+      </c>
+      <c r="E3" s="21" t="inlineStr">
+        <is>
+          <t>AfDB; DBSA; Absa Capital; Barclays/ABSA Group</t>
+        </is>
+      </c>
+      <c r="F3" s="21" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="G3" s="21" t="inlineStr">
+        <is>
+          <t>Pan-Africa</t>
+        </is>
+      </c>
+      <c r="H3" s="21" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="I3" s="21" t="inlineStr">
+        <is>
+          <t>AfDB says target up to USD 450m initially; DBSA annual report says first close in Sep 2007 at USD 625m and DBSA committed USD 100m.</t>
+        </is>
+      </c>
+      <c r="J3" s="21" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="K3" s="21" t="inlineStr">
+        <is>
+          <t>Add to Commitments and Fund Vehicles if historical scope includes older infrastructure funds; likely multiple African PF/SWF LP rows or a single aggregate historical PAIDF row.</t>
+        </is>
+      </c>
+      <c r="L3" s="21" t="inlineStr">
+        <is>
+          <t>AfDB page names PIC/GEPF and EPPF as potential/reputable investors and PIC as chief sponsor; DBSA annual report says DBSA invested alongside PIC, AfDB, and SSNIT.</t>
+        </is>
+      </c>
+      <c r="M3" s="21" t="inlineStr">
+        <is>
+          <t>https://www.afdb.org/en/news-and-events/pan-african-infrastructure-development-fund-paidf-afdb-group-proposes-us-50-million-investment-in-paidf-3476</t>
+        </is>
+      </c>
+      <c r="N3" s="21" t="inlineStr">
+        <is>
+          <t>https://www.dbsa.org/sites/default/files/media/documents/2021-09/DBSA%20and%20Development%20Fund%20Annual%20Reports%202008.pdf</t>
+        </is>
+      </c>
+      <c r="O3" s="21" t="inlineStr">
+        <is>
+          <t>PIC/GEPF + DFI sweep</t>
+        </is>
+      </c>
+      <c r="P3" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>Candidate - new 2026 item</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Hlayisani Venture Fund II (HVF II)</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>Hlayisani Capital</t>
+        </is>
+      </c>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>Public Investment Corporation (PIC)</t>
+        </is>
+      </c>
+      <c r="E4" s="21" t="inlineStr">
+        <is>
+          <t>SA SME Fund; additional private investors and family offices</t>
+        </is>
+      </c>
+      <c r="F4" s="21" t="inlineStr">
+        <is>
+          <t>VC / technology-enabled SMEs</t>
+        </is>
+      </c>
+      <c r="G4" s="21" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="H4" s="21" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I4" s="21" t="inlineStr">
+        <is>
+          <t>R500m / about USD 30m commitments to date; final close targeted June 2026.</t>
+        </is>
+      </c>
+      <c r="J4" s="21" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="K4" s="21" t="inlineStr">
+        <is>
+          <t>Add to Commitments and Fund Vehicles as confirmed first-close/commitments-to-date, with note that final close is pending.</t>
+        </is>
+      </c>
+      <c r="L4" s="21" t="inlineStr">
+        <is>
+          <t>Hlayisani and multiple trade sources say Fund II is anchored by PIC and SA SME Fund with R500m committed to date.</t>
+        </is>
+      </c>
+      <c r="M4" s="21" t="inlineStr">
+        <is>
+          <t>https://hlayisani.com/</t>
+        </is>
+      </c>
+      <c r="N4" s="21" t="inlineStr">
+        <is>
+          <t>https://disruptafrica.com/2026/03/11/sas-hlayisani-capital-launches-2nd-fund-with-initial-29-9m-in-commitments/</t>
+        </is>
+      </c>
+      <c r="O4" s="21" t="inlineStr">
+        <is>
+          <t>PIC/GEPF + recent fund-close sweep</t>
+        </is>
+      </c>
+      <c r="P4" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>Candidate - research vehicle identity</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>Medu Capital Fund II</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>Medu Capital</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>Eskom Pension and Provident Fund; Public Investment Corporation</t>
+        </is>
+      </c>
+      <c r="E5" s="21" t="inlineStr">
+        <is>
+          <t>DBSA; CDC Group; FMO; Alternative Equity Partners; Brait; Metropolitan; Vunani</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="inlineStr">
+        <is>
+          <t>PE / BEE mid-market</t>
+        </is>
+      </c>
+      <c r="G5" s="21" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="H5" s="21" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="I5" s="21" t="inlineStr">
+        <is>
+          <t>DBSA annual report says capitalisation R850m; DBSA provided R100m.</t>
+        </is>
+      </c>
+      <c r="J5" s="21" t="inlineStr">
+        <is>
+          <t>M-H</t>
+        </is>
+      </c>
+      <c r="K5" s="21" t="inlineStr">
+        <is>
+          <t>Review whether the vehicle is in scope as alternatives/fund LP; likely add if historical South Africa domestic PE vehicles are included.</t>
+        </is>
+      </c>
+      <c r="L5" s="21" t="inlineStr">
+        <is>
+          <t>DBSA annual report identifies Medu II investors including EPPF, PIC, CDC, FMO and DBSA.</t>
+        </is>
+      </c>
+      <c r="M5" s="21" t="inlineStr">
+        <is>
+          <t>https://www.dbsa.org/sites/default/files/media/documents/2021-09/DBSA%20and%20Development%20Fund%20Annual%20Reports%202008.pdf</t>
+        </is>
+      </c>
+      <c r="N5" s="21" t="inlineStr"/>
+      <c r="O5" s="21" t="inlineStr">
+        <is>
+          <t>DBSA historical PE fund sweep</t>
+        </is>
+      </c>
+      <c r="P5" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F179"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
@@ -9868,7 +10315,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10290,7 +10737,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11166,7 +11613,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Clarify Oyass and Wessal vehicle labels
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -2294,7 +2294,7 @@
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Oyass Capital</t>
+          <t>Oyass Capital (SME fund)</t>
         </is>
       </c>
       <c r="D7" s="23" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="G7" s="23" t="inlineStr">
         <is>
-          <t>Column H identifies a named African PF/SWF, a named cohort, or the allocator itself is an African SWF/PF vehicle.</t>
+          <t>Retain as a fund/financing vehicle, not a GP. FONSIS describes Oyass Capital as an SME private-equity fund/financing vehicle; SEAF is the manager.</t>
         </is>
       </c>
       <c r="H7" s="23" t="inlineStr"/>
@@ -3170,7 +3170,7 @@
       </c>
       <c r="C31" s="23" t="inlineStr">
         <is>
-          <t>Wessal Capital</t>
+          <t>Wessal Capital (SWF joint investment vehicle)</t>
         </is>
       </c>
       <c r="D31" s="23" t="inlineStr">
@@ -3190,10 +3190,14 @@
       </c>
       <c r="G31" s="23" t="inlineStr">
         <is>
-          <t>Column H identifies a named African PF/SWF, a named cohort, or the allocator itself is an African SWF/PF vehicle.</t>
-        </is>
-      </c>
-      <c r="H31" s="23" t="inlineStr"/>
+          <t>Retain as a direct SWF joint investment vehicle/platform rather than a conventional GP-managed fund. Ithmar names Wessal as an investment vehicle and identifies Wessal Bouregreg and Wessal Casa-Port as launched projects.</t>
+        </is>
+      </c>
+      <c r="H31" s="23" t="inlineStr">
+        <is>
+          <t>https://www.ithmar.gov.ma/en/our-portfolio/</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="23" t="inlineStr">
@@ -4570,7 +4574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F179"/>
+  <dimension ref="A1:F180"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="16" min="1" max="2"/>
@@ -5408,7 +5412,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>FONSIS Oyass Capital launch with SEAF as manager</t>
+          <t>Oyass Capital as FONSIS/KfW/World Bank-backed SME fund/financing vehicle; management mandate awarded to SEAF</t>
         </is>
       </c>
     </row>
@@ -10305,6 +10309,38 @@
       <c r="F179" t="inlineStr">
         <is>
           <t>PIC/GEPF LP confirmation in Africa Food Security Fund; co-investors AfDB, CDC/BII, DGGF, IFU, EBID and Kuramo</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Ithmar Capital</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>SWF portfolio page</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Ithmar Capital - Our portfolio: Wessal</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>https://www.ithmar.gov.ma/en/our-portfolio/</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Wessal as SWF joint investment vehicle; EUR 2.5bn equity commitment; projects Wessal Bouregreg and Wessal Casa-Port</t>
         </is>
       </c>
     </row>
@@ -10340,6 +10376,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="16">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -10763,6 +10800,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="23.25" customHeight="1" s="16">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -11637,6 +11675,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="16">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -11644,6 +11683,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="23.25" customHeight="1" s="16">
       <c r="A5" s="1" t="inlineStr">
         <is>
@@ -11752,6 +11792,8 @@
         <v>0.19</v>
       </c>
     </row>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="16">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -12025,6 +12067,8 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
+    <row r="31"/>
     <row r="32" ht="15" customHeight="1" s="16">
       <c r="A32" s="8" t="inlineStr">
         <is>
@@ -23647,6 +23691,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="23.25" customHeight="1" s="16">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -27157,22 +27202,22 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Fund LP</t>
+          <t>Platform / direct strategic investment vehicle</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Wessal Capital</t>
+          <t>Wessal Capital joint venture</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Wessal Capital (joint Morocco + Gulf SWFs platform)</t>
+          <t>Wessal Capital (SWF joint investment vehicle)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Direct / Real estate, infra</t>
+          <t>Direct / real estate / tourism infrastructure</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -27187,7 +27232,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>USD 2.5bn target</t>
+          <t>EUR 2.5bn equity commitment</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -27202,7 +27247,7 @@
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>Wessal Capital announcements</t>
+          <t>Ithmar portfolio: Wessal</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
@@ -27212,7 +27257,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>Joint platform with Abu Dhabi, Kuwait, Qatar SWFs.</t>
+          <t>Ithmar describes Wessal as an investment vehicle / joint venture equally owned by five SWFs, not a conventional GP-managed fund. Named projects include Wessal Bouregreg and Wessal Casa-Port.</t>
         </is>
       </c>
     </row>
@@ -28450,7 +28495,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Fund LP</t>
+          <t>Fund LP / sponsor</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -28460,7 +28505,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Oyass Capital</t>
+          <t>Oyass Capital (SME fund)</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -28503,7 +28548,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>FONSIS partnered with KfW (Germany) to launch Oyass Capital for Senegalese SMEs; awarded mgmt mandate to SEAF after intl tender.</t>
+          <t>FONSIS and KfW/World Bank launched Oyass Capital as an SME-focused private-equity fund/financing vehicle; FONSIS says SEAF received the management mandate after an international tender.</t>
         </is>
       </c>
     </row>
@@ -33230,6 +33275,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="45.75" customHeight="1" s="16">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -33529,12 +33575,12 @@
     <row r="8" ht="34.5" customHeight="1" s="16">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Oyass Capital</t>
+          <t>Oyass Capital (SME fund)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>SEAF (Small Enterprise Assistance Funds)</t>
+          <t>SEAF / SEAF Senegal</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -33544,7 +33590,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>~82 (XOF 50bn)</t>
+          <t>~79m target / EUR 54m mobilized</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -33580,7 +33626,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>FONSIS + KfW launch; SEAF mandate award after international tender.</t>
+          <t>FONSIS source describes Oyass Capital as an SME-focused private-equity fund/financing vehicle set up with KfW/World Bank support; management mandate awarded to SEAF.</t>
         </is>
       </c>
     </row>
@@ -34519,12 +34565,12 @@
     <row r="25" ht="34.5" customHeight="1" s="16">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Wessal Capital</t>
+          <t>Wessal Capital (SWF joint investment vehicle)</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Wessal Capital partnership</t>
+          <t>Wessal Capital joint venture</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -34534,12 +34580,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>USD 2.5bn target</t>
+          <t>EUR 2.5bn equity commitment</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Direct (real estate / infra)</t>
+          <t>Direct / real estate / tourism infrastructure</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -34565,12 +34611,12 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Abu Dhabi, Kuwait, Qatar SWFs (Gulf SWF co-investors)</t>
+          <t>Al Ajial Investment Fund Holding; Mubadala; Public Investment Fund; Qatar Holding</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Joint Morocco + Gulf SWF platform.</t>
+          <t>Ithmar describes Wessal as a joint investment vehicle, equally owned by five SWFs. Specific launched projects: Wessal Bouregreg and Wessal Casa-Port.</t>
         </is>
       </c>
     </row>
@@ -35135,6 +35181,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="45.75" customHeight="1" s="16">
       <c r="A3" s="24" t="inlineStr">
         <is>
@@ -35976,6 +36023,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="23.25" customHeight="1" s="16">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -37650,6 +37698,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="15" customHeight="1" s="16">
       <c r="A19" s="18" t="inlineStr">
         <is>
@@ -37665,6 +37714,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Classify fund of funds separately
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -29274,7 +29274,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Fund of funds (PE / VC / Private credit)</t>
+          <t>Fund of Funds</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -29349,7 +29349,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Fund of funds (PE / VC / Private credit)</t>
+          <t>Fund of Funds</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -32298,7 +32298,7 @@
       </c>
       <c r="G4" s="26" t="inlineStr">
         <is>
-          <t>FoF (PE/VC/Private credit)</t>
+          <t>Fund of Funds</t>
         </is>
       </c>
       <c r="H4" s="26" t="inlineStr">
@@ -33475,7 +33475,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>FoF (PE/VC/Private credit)</t>
+          <t>Fund of Funds</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add NSIA fund and healthcare commitments
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -2044,7 +2044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="16" min="1" max="1"/>
@@ -4121,6 +4121,216 @@
       <c r="H57" t="inlineStr">
         <is>
           <t>https://english.dggf.nl/latest/news/2019/01/24/zebu-s-africa-food-security-fund-a-dggf-investee-reaches-total-fund-size-of-usd-84-million</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Funds &amp; LP Co-Investors</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>added May 2026</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Alitheia IDF Fund</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>NSIA Nigeria</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Column H identifies NSIA, an African SWF, as a named LP/sponsor in the vehicle.</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://nsia.com.ng/the-nsia-model-catalyzing-development-through-sustainable-investments/</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Funds &amp; LP Co-Investors</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>added May 2026</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Ingressive Capital Fund / funds</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>NSIA Nigeria</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Column H identifies NSIA, an African SWF, as a named LP/sponsor in the vehicle.</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://nsia.com.ng/the-nsia-model-catalyzing-development-through-sustainable-investments/</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Funds &amp; LP Co-Investors</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>added May 2026</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Verod Growth Fund II</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>NSIA Nigeria</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Column H identifies NSIA, an African SWF, as a named LP/sponsor in the vehicle.</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://nsia.com.ng/the-nsia-model-catalyzing-development-through-sustainable-investments/</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Funds &amp; LP Co-Investors</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>added May 2026</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Verod Growth Fund III</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>NSIA Nigeria</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Column H identifies NSIA, an African SWF, as a named LP/sponsor in the vehicle.</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://nsia.com.ng/the-nsia-model-catalyzing-development-through-sustainable-investments/</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Funds &amp; LP Co-Investors</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>added May 2026</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>MedServe oncology and diagnostics expansion</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>NSIA Nigeria</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Column H identifies NSIA, an African SWF, as a named LP/sponsor in the vehicle.</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>https://www.ifc.org/en/pressroom/2026/ifc-and-nsia-to-scale-oncology-and-diagnostic-services-for-underserved-communities</t>
         </is>
       </c>
     </row>
@@ -4574,7 +4784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F180"/>
+  <dimension ref="A1:F186"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="16" min="1" max="2"/>
@@ -10341,6 +10551,198 @@
       <c r="F180" t="inlineStr">
         <is>
           <t>Wessal as SWF joint investment vehicle; EUR 2.5bn equity commitment; projects Wessal Bouregreg and Wessal Casa-Port</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>NSIA</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Press release / sustainability article</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>The NSIA Model: Catalyzing Development Through Sustainable Investments</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>https://nsia.com.ng/the-nsia-model-catalyzing-development-through-sustainable-investments/</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>NSIA investments in Alitheia IDF, Ingressive Capital and Verod Capital; MedServe impact reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>NSIA</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Impact report</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>NSIA Development Impact Report 2021</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>https://nsia.com.ng/download/56/2021-report/10080/nsia-development-impact-report-2021_.pdf</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Verod Growth Fund II USD 5m commitment and Verod Growth Fund III USD 7.5m commitment</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>IFC / NSIA</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Press release</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>IFC and NSIA to Scale Oncology and Diagnostic Services for Underserved Communities in Nigeria</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>https://www.ifc.org/en/pressroom/2026/ifc-and-nsia-to-scale-oncology-and-diagnostic-services-for-underserved-communities</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>MedServe expansion project size USD 154.1m; IFC USD 24.5m local-currency financing</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Alitheia IDF</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Investor profile</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Soros Economic Development Fund - Alitheia IDF Fund LP</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>https://www.soroseconomicdevelopmentfund.org/investments/alitheia-idf-fund-lp</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Alitheia IDF as USD 100m gender-lens fund and SEDF co-investor</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Ingressive Capital</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Manager profile</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Ingressive Capital - About Us</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>https://ingressivecapital.com/about-us/</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Ingressive Capital strategy and geographic focus</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Verod Capital</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Manager profile</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Verod Capital - Home</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>https://www.verod.com/</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Verod Growth fund manager profile and AUM context</t>
         </is>
       </c>
     </row>
@@ -10376,7 +10778,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="16">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -10800,7 +11201,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="23.25" customHeight="1" s="16">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -11675,7 +12075,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="16">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -11683,7 +12082,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="23.25" customHeight="1" s="16">
       <c r="A5" s="1" t="inlineStr">
         <is>
@@ -11792,8 +12190,6 @@
         <v>0.19</v>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="16">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -12067,8 +12463,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32" ht="15" customHeight="1" s="16">
       <c r="A32" s="8" t="inlineStr">
         <is>
@@ -23691,7 +24085,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="23.25" customHeight="1" s="16">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -25331,7 +25724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O87"/>
+  <dimension ref="A1:O92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="16" min="1" max="1"/>
@@ -31965,11 +32358,387 @@
         </is>
       </c>
     </row>
-    <row r="88" ht="45.75" customHeight="1" s="16"/>
-    <row r="89" ht="34.5" customHeight="1" s="16"/>
-    <row r="90" ht="34.5" customHeight="1" s="16"/>
-    <row r="91" ht="23.25" customHeight="1" s="16"/>
-    <row r="92" ht="23.25" customHeight="1" s="16"/>
+    <row r="88" ht="45.75" customHeight="1" s="16">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Nigeria Sovereign Investment Authority (NSIA)</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>SWF (FGF)</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Alitheia Capital / IDF Capital</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Alitheia IDF Fund</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>PE / gender-lens</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>2021 or earlier</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Not disclosed publicly</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>NSIA sustainability disclosure</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>NSIA sustainability article Apr 2026</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>NSIA names Alitheia IDF among investments supporting women-led and women-impacting businesses. Specific NSIA ticket size not publicly disclosed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="34.5" customHeight="1" s="16">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Nigeria Sovereign Investment Authority (NSIA)</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>SWF (FGF)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Ingressive Capital</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Ingressive Capital Fund / funds</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>VC / technology-enabled SMEs</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Africa / Nigeria-led</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>2023 or earlier</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Not disclosed publicly</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>NSIA sustainability disclosure</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>NSIA sustainability article Apr 2026</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>NSIA names Ingressive Capital among investments supporting women-led and women-impacting businesses. Public NSIA source does not identify a specific vintage, so retained as platform/fund exposure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="34.5" customHeight="1" s="16">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Nigeria Sovereign Investment Authority (NSIA)</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>SWF (FGF)</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Verod Capital Management</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Verod Growth Fund II</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>PE / growth equity</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>West Africa / Nigeria</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>2017</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>USD 5m</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>NSIA impact report</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>NSIA Development Impact Report 2021</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>NSIA impact report states the Authority invested USD 5m in Verod Growth Fund II in 2017.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="23.25" customHeight="1" s="16">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Nigeria Sovereign Investment Authority (NSIA)</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>SWF (FGF)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Verod Capital Management</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Verod Growth Fund III</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>PE / growth equity</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>West Africa / Nigeria</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>2021 or earlier</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>USD 7.5m commitment</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>NSIA impact report</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>NSIA Development Impact Report 2021</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>NSIA impact report states the Authority subsequently invested in Verod Growth Fund III, with 8% of the USD 7.5m commitment disbursed at the time of reporting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="23.25" customHeight="1" s="16">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Nigeria Sovereign Investment Authority (NSIA)</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>SWF (healthcare subsidiary)</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Direct / co-investment</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>NSIA Advanced Medical Services Limited (MedServe)</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>MedServe oncology and diagnostics expansion</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Direct / Healthcare</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>2026</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>USD 154.1m project; IFC USD 24.5m local-currency financing</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>IFC press release</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>IFC-NSIA MedServe financing Feb 2026</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>IFC and NSIA partnered to finance MedServe, NSIA's wholly owned healthcare subsidiary, to scale diagnostic centers, cancer care facilities and cath labs across Nigerian states.</t>
+        </is>
+      </c>
+    </row>
     <row r="93" ht="124.5" customHeight="1" s="16"/>
     <row r="94" ht="124.5" customHeight="1" s="16"/>
     <row r="95" ht="79.5" customHeight="1" s="16"/>
@@ -33251,7 +34020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="16" min="1" max="1"/>
@@ -33275,7 +34044,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="45.75" customHeight="1" s="16">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -35136,11 +35904,264 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="23.25" customHeight="1" s="16"/>
-    <row r="36" ht="15" customHeight="1" s="16"/>
-    <row r="37" ht="34.5" customHeight="1" s="16"/>
-    <row r="38" ht="23.25" customHeight="1" s="16"/>
-    <row r="39" ht="34.5" customHeight="1" s="16"/>
+    <row r="35" ht="23.25" customHeight="1" s="16">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Alitheia IDF Fund</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Alitheia Capital / IDF Capital</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2021 or earlier</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>PE / gender-lens</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>NSIA Nigeria</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Soros Economic Development Fund</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>NSIA names Alitheia IDF as an investment; SEDF describes Alitheia IDF as a USD 100m gender-lens fund. NSIA ticket size not disclosed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1" s="16">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Ingressive Capital Fund / funds</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Ingressive Capital</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2023 or earlier</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>VC / technology-enabled SMEs</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Africa / Nigeria-led</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>NSIA Nigeria</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>NSIA names Ingressive Capital as an investment; specific NSIA vehicle/vintage and ticket size not publicly disclosed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="34.5" customHeight="1" s="16">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Verod Growth Fund II</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Verod Capital Management</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>PE / growth equity</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>West Africa / Nigeria</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>NSIA Nigeria (USD 5m)</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>NSIA impact report identifies a USD 5m FGF commitment to Verod Growth Fund II.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="23.25" customHeight="1" s="16">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Verod Growth Fund III</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Verod Capital Management</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2021 or earlier</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>PE / growth equity</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>West Africa / Nigeria</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>NSIA Nigeria (USD 7.5m commitment)</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>NSIA impact report identifies a USD 7.5m FGF commitment to Verod Growth Fund III.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="34.5" customHeight="1" s="16">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>MedServe oncology and diagnostics expansion</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>NSIA Advanced Medical Services Limited (MedServe)</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>154.1 project size</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Direct / Healthcare</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>NSIA Nigeria</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>1</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>International Development Association Private Sector Window Local Currency Facility</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>IFC provided roughly NGN 14.2bn / USD 24.5m local-currency financing for NSIA's wholly owned MedServe expansion program.</t>
+        </is>
+      </c>
+    </row>
     <row r="40" ht="34.5" customHeight="1" s="16"/>
     <row r="41" ht="15" customHeight="1" s="16"/>
     <row r="42" ht="45.75" customHeight="1" s="16"/>
@@ -35181,7 +36202,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="45.75" customHeight="1" s="16">
       <c r="A3" s="24" t="inlineStr">
         <is>
@@ -36023,7 +37043,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="23.25" customHeight="1" s="16">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -37698,7 +38717,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="15" customHeight="1" s="16">
       <c r="A19" s="18" t="inlineStr">
         <is>
@@ -37714,7 +38732,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add NSIA InfraCredit vehicles
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -2044,7 +2044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="16" min="1" max="1"/>
@@ -4331,6 +4331,90 @@
       <c r="H62" t="inlineStr">
         <is>
           <t>https://www.ifc.org/en/pressroom/2026/ifc-and-nsia-to-scale-oncology-and-diagnostic-services-for-underserved-communities</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Funds &amp; LP Co-Investors</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>added May 2026</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>InfraCredit</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>NSIA Nigeria</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Column H identifies NSIA, an African SWF, as sponsor/anchor investor; InfraCredit also has named Nigerian pension shareholders.</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>https://nsia.com.ng/portfolio/infracredit/</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Funds &amp; LP Co-Investors</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>added May 2026</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Construction Finance Warehouse Facility (CFWF)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>NSIA Nigeria</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Column H identifies NSIA, an African SWF, as sponsor/anchor investor; InfraCredit also has named Nigerian pension shareholders.</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>https://infracredit.ng/nsia-invests-ngn10-billion-into-an-innovative-construction-finance-warehouse-facility-in-collaboration-with-infracredit-to-support-bankable-greenfield-infrastructure-project-finance-in-nigeria/</t>
         </is>
       </c>
     </row>
@@ -4784,7 +4868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F186"/>
+  <dimension ref="A1:F192"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="16" min="1" max="2"/>
@@ -10743,6 +10827,198 @@
       <c r="F186" t="inlineStr">
         <is>
           <t>Verod Growth fund manager profile and AUM context</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>InfraCredit</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Case study</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Harvard Business School - InfraCredit and the Project Inception Facility</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>https://www.hbs.edu/faculty/Pages/item.aspx?num=66419</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>InfraCredit business model and project-inception funding context</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>InfraCredit</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>NSIA portfolio page</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>NSIA Portfolio - InfraCredit</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>https://nsia.com.ng/portfolio/infracredit/</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>InfraCredit as NSIA/GuarantCo participant vehicle catalysing pension and insurance investment</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>InfraCredit / NSIA</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Press release</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>NSIA invests NGN10bn into Construction Finance Warehouse Facility with InfraCredit</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>https://infracredit.ng/nsia-invests-ngn10-billion-into-an-innovative-construction-finance-warehouse-facility-in-collaboration-with-infracredit-to-support-bankable-greenfield-infrastructure-project-finance-in-nigeria/</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>NSIA NGN10bn anchor investment; CFWF target NGN100bn capacity; InfraCredit capitalization USD237m+</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>InfraCredit</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Press release</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>KfW Development Bank invests EUR31m subordinated capital in InfraCredit</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>https://infracredit.ng/kfw-development-bank-invests-e31-million-surbordinated-capital-in-infracredit/</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>KfW subordinated capital and InfraCredit establishment by NSIA with GuarantCo/PIDG</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>InfraCredit</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>OECD case study</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>InfraCredit: Making infrastructure projects in Nigeria more bankable through credit enhancement</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>https://www.oecd.org/en/publications/blended-finance-case-studies_2fb90b9a-en/infracredit-making-infrastructure-projects-in-nigeria-more-bankable-through-credit-enhancement_bdb679c6-en.html</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>PIDG/NSIA establishment, GuarantCo initial contingent capital, InfraCo Africa and domestic institutional mobilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>NSIA</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Financial statements</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>NSIA 2025 Group Financial Statements - InfraCredit ownership</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>https://nsia.com.ng/download/267/2025-report/15287/nsia-2025-group-financial-statements-usd.pdf</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>NSIA retained InfraCredit ownership interest; Access ARM Pensions, CardinalStone, AFC and insurers as shareholders</t>
         </is>
       </c>
     </row>
@@ -25724,7 +26000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O92"/>
+  <dimension ref="A1:O94"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="16" min="1" max="1"/>
@@ -32739,8 +33015,158 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="124.5" customHeight="1" s="16"/>
-    <row r="94" ht="124.5" customHeight="1" s="16"/>
+    <row r="93" ht="124.5" customHeight="1" s="16">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Nigeria Sovereign Investment Authority (NSIA)</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>SWF (NIF sub-fund)</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Platform / direct strategic investment vehicle</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Infrastructure Credit Guarantee Company PLC (InfraCredit)</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>InfraCredit</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Infrastructure credit enhancement / guarantees</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>2016/2017</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>43.88% ownership interest retained by NSIA at FY2025; capitalization over USD 237m reported in 2023</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>NSIA portfolio / financial statements</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>NSIA InfraCredit portfolio; NSIA FY2025 financial statements</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>InfraCredit is a specialised infrastructure credit enhancement facility established by NSIA with GuarantCo/PIDG. NSIA FY2025 statements report a 43.88% retained ownership interest after shareholder changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="124.5" customHeight="1" s="16">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Nigeria Sovereign Investment Authority (NSIA)</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>SWF (NIF sub-fund)</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Direct / facility anchor</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>InfraCredit</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Construction Finance Warehouse Facility (CFWF)</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Infrastructure construction finance / credit enhancement</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>2023</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>NGN 10bn NSIA anchor; target NGN 100bn facility capacity</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>NGN</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>InfraCredit press release</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>InfraCredit CFWF announcement Oct 2023</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>NSIA invested NGN 10bn into a multi-funder revolving construction finance facility developed with InfraCredit to support greenfield infrastructure projects backed by InfraCredit guarantees.</t>
+        </is>
+      </c>
+    </row>
     <row r="95" ht="79.5" customHeight="1" s="16"/>
     <row r="96" ht="34.5" customHeight="1" s="16"/>
     <row r="97" ht="45.75" customHeight="1" s="16"/>
@@ -34020,7 +34446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="16" min="1" max="1"/>
@@ -35946,7 +36372,6 @@
       <c r="I35" t="n">
         <v>0</v>
       </c>
-      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
           <t>Soros Economic Development Fund</t>
@@ -36000,8 +36425,6 @@
       <c r="I36" t="n">
         <v>0</v>
       </c>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
           <t>NSIA names Ingressive Capital as an investment; specific NSIA vehicle/vintage and ticket size not publicly disclosed.</t>
@@ -36048,8 +36471,6 @@
       <c r="I37" t="n">
         <v>0</v>
       </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
           <t>NSIA impact report identifies a USD 5m FGF commitment to Verod Growth Fund II.</t>
@@ -36098,8 +36519,6 @@
       <c r="I38" t="n">
         <v>0</v>
       </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
           <t>NSIA impact report identifies a USD 7.5m FGF commitment to Verod Growth Fund III.</t>
@@ -36162,8 +36581,112 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="34.5" customHeight="1" s="16"/>
-    <row r="41" ht="15" customHeight="1" s="16"/>
+    <row r="40" ht="34.5" customHeight="1" s="16">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>InfraCredit</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Infrastructure Credit Guarantee Company PLC</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2016/2017</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>USD 237m+ capitalization reported in 2023</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Infrastructure credit enhancement / guarantees</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>3</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>NSIA Nigeria; Access ARM Pensions; CardinalStone Pensions</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>4</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>GuarantCo / PIDG; KfW; AfDB; InfraCo Africa</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Africa Finance Corporation; Leadway Assurance; AIICO Insurance; FCDO / Mobilist</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>NSIA established InfraCredit with GuarantCo/PIDG. Later shareholders/backers include KfW, AfDB, InfraCo Africa, AFC, insurers, and Nigerian pension shareholders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15" customHeight="1" s="16">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Construction Finance Warehouse Facility (CFWF)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>InfraCredit / NSIA</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>NGN 10bn anchor; NGN 100bn target capacity</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Infrastructure construction finance / credit enhancement</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>NSIA Nigeria</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>NSIA provided NGN 10bn anchor funding; FSD Africa supported facility set-up costs through technical assistance rather than a disclosed LP/co-investment commitment.</t>
+        </is>
+      </c>
+    </row>
     <row r="42" ht="45.75" customHeight="1" s="16"/>
     <row r="43" ht="45.75" customHeight="1" s="16"/>
     <row r="44" ht="57" customHeight="1" s="16"/>
@@ -36185,7 +36708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="16" min="1" max="1"/>
@@ -36261,11 +36784,11 @@
         </is>
       </c>
       <c r="B5" s="23" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C5" s="23" t="inlineStr">
         <is>
-          <t>AfricInvest FIVE (Financial Inclusion Vehicle); Africa50 (general); Africa50 Infrastructure Acceleration Fund (IAF); Mediterrania Capital II / III / IV; Nigeria Infrastructure Fund (NIF, NSIA sub-fund); Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Africa Food Security Fund (AFSF)</t>
+          <t>AfricInvest FIVE (Financial Inclusion Vehicle); Africa50 (general); Africa50 Infrastructure Acceleration Fund (IAF); Mediterrania Capital II / III / IV; Nigeria Infrastructure Fund (NIF, NSIA sub-fund); Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Africa Food Security Fund (AFSF); InfraCredit</t>
         </is>
       </c>
       <c r="D5" s="23" t="inlineStr">
@@ -36461,11 +36984,11 @@
         </is>
       </c>
       <c r="B13" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>AfricInvest FIVE (Financial Inclusion Vehicle); Oyass Capital</t>
+          <t>AfricInvest FIVE (Financial Inclusion Vehicle); Oyass Capital; InfraCredit</t>
         </is>
       </c>
       <c r="D13" s="23" t="inlineStr">
@@ -36991,6 +37514,56 @@
         </is>
       </c>
       <c r="E50" t="inlineStr">
+        <is>
+          <t>3 (Selective / TA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>GuarantCo / PIDG</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>InfraCredit</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Guarantee/catalytic capital provider that established InfraCredit with NSIA via PIDG/GuarantCo.</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>3 (Selective / TA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>InfraCo Africa</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>InfraCredit</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>PIDG project-development arm/shareholder capital provider to InfraCredit.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>3 (Selective / TA)</t>
         </is>

</xml_diff>

<commit_message>
Add VCTF Ghana Oasis commitments
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -2044,7 +2044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="16" min="1" max="1"/>
@@ -4415,6 +4415,46 @@
       <c r="H64" t="inlineStr">
         <is>
           <t>https://infracredit.ng/nsia-invests-ngn10-billion-into-an-innovative-construction-finance-warehouse-facility-in-collaboration-with-infracredit-to-support-bankable-greenfield-infrastructure-project-finance-in-nigeria/</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Funds &amp; LP Co-Investors</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>42</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Oasis Africa VC Fund (OAF)</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Venture Capital Trust Fund (VCTF)</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>VCTF is a Ghanaian government-backed venture capital fund of funds; VCTF 2015 annual report confirms USD 2m commitment and DGGF research confirms the fund was locally domiciled to access VCTF co-investment.</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>https://vctf.com.gh/wp-content/uploads/2022/09/Venture-Capital-Annual-report-2015.pdf; https://english.dggf.nl/site/binaries/site-content/collections/documents/2025/11/17/getting-sme-risk-capital-funds-to-first-close/dggf-knowledge-product-getting-sme-risk-capital-funds-to-first-close.pdf</t>
         </is>
       </c>
     </row>
@@ -4868,7 +4908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F192"/>
+  <dimension ref="A1:F199"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="16" min="1" max="2"/>
@@ -11019,6 +11059,230 @@
       <c r="F192" t="inlineStr">
         <is>
           <t>NSIA retained InfraCredit ownership interest; Access ARM Pensions, CardinalStone, AFC and insurers as shareholders</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>VCTF Ghana / Oasis Capital</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Media / impact report coverage</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Graphic Online - Venture Capital Fund invests over GHc359m in local businesses</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>https://www.graphic.com.gh/news/general-news/ghana-news-venture-capital-fund-invests-over-ghc359m-in-local-businesses.html</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>VCTF impact report coverage; GHc359.6m invested, GHc2bn leveraged; Oasis Capital and Injaro Ghana Venture Fund identified as anchored/impactful funds</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Oasis Africa VC Fund</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>DFI research report</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>DGGF - Getting SME Risk Capital Funds to First Close</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>https://english.dggf.nl/site/binaries/site-content/collections/documents/2025/11/17/getting-sme-risk-capital-funds-to-first-close/dggf-knowledge-product-getting-sme-risk-capital-funds-to-first-close.pdf</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Oasis Africa VC Fund Ghana domicile, VCTF government co-investment rationale, DGGF legal TA and subsequent DFI crowd-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Oasis Africa VC Fund</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>DFI announcement</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>DGGF - Oasis Capital Ghana first close Oasis Africa VC Fund USD 27 million</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>https://english.dggf.nl/latest/news/2018/5/31/oasis-capital-ghana-first-close-oasis-africa-vc-fund-usd-27-million</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>OAF first close amount and DGGF role</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Oasis Africa VC Fund</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>GP announcement</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Oasis Capital Ghana - Oasis Africa VC Fund first close</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>https://oasiscapitalghana.com/v2/oasis-capital-ghana-has-completed-the-first-close-of-its-second-fund-oasis-africa-vc-fund-oaf/</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>OAF first close: USD 27m, DGGF USD 5m, IFC USD 7m and local investor base over USD 15m</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Oasis Africa VC Fund</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>DFI fund profile</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>EIB - Oasis Africa SME Fund</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>https://www.eib.org/en/products/equity/funds/oasis-africa-sme-fund</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Oasis Africa VC Fund final fund size USD 50.5m and EIB USD 8m commitment</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>VCTF Ghana / Oasis Capital</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Allocator annual report</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Venture Capital Trust Fund - Annual Report 2015</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>https://vctf.com.gh/wp-content/uploads/2022/09/Venture-Capital-Annual-report-2015.pdf</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>VCTF USD 2m commitment to Oasis Africa Fund Limited and Ebankese Venture Fund portfolio context</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>VCTF Ghana</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Allocator profile</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Venture Capital Trust Fund - About Us</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>https://vctf.com.gh/about-us/</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>VCTF mandate as government-backed venture capital fund of funds focused on SME venture funds</t>
         </is>
       </c>
     </row>
@@ -26000,7 +26264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O94"/>
+  <dimension ref="A1:O97"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="16" min="1" max="1"/>
@@ -33167,9 +33431,233 @@
         </is>
       </c>
     </row>
-    <row r="95" ht="79.5" customHeight="1" s="16"/>
-    <row r="96" ht="34.5" customHeight="1" s="16"/>
-    <row r="97" ht="45.75" customHeight="1" s="16"/>
+    <row r="95" ht="79.5" customHeight="1" s="16">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Venture Capital Trust Fund (VCTF) Ghana</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Government-backed VC fund of funds</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Fund LP / Anchor</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Oasis Capital Ghana</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Oasis Africa VC Fund (OAF)</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>PE / SME / VC</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Ghana + Cote d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>2015/2016</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>USD 2m VCTF commitment; OAF first close USD 27m; final/target size ~USD 50m</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>Annual report / DFI report / fund announcement</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>VCTF 2015 Annual Report; DGGF Oasis first-close announcement; DGGF catalytic-capital paper</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>VCTF 2015 annual report states VCTF made a USD 2m commitment to Oasis Africa Fund Limited, Oasis Capital Partners second fund. DGGF later described OAF as Ghana-domiciled to access VCTF government co-investment and noted the structure helped crowd in international DFIs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="34.5" customHeight="1" s="16">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Venture Capital Trust Fund (VCTF) Ghana</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Government-backed VC fund of funds</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Fund LP / Anchor</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Mirepa Investment Advisors</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Mirepa Capital SME Fund I</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>PE / SME growth</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>2023</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Part of GHS 120m initial close / reported USD 10.5m VCTF-led investment</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>GHS / USD</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>Press / trade press</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>Mirepa initial-close sources; Afrikan Heroes VCTF lead role</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>VCTF is named in the Mirepa LP group alongside Petra Trust, Axis Pensions and CAMCOL-managed pension schemes; public coverage describes VCTF as leading the investment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="45.75" customHeight="1" s="16">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Venture Capital Trust Fund (VCTF) Ghana</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Government-backed VC fund of funds</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Fund LP / Anchor</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Injaro Investment Advisors</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Injaro Ghana Venture Capital Fund (IGVCF)</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>PE / SME / VC</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Ghana + Cote d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>2023</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Part of GHS 216m final close; VCTF participation disclosed</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>GHS</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>Press / impact-report coverage</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>Injaro final-close sources; Graphic VCTF impact-report coverage</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>VCTF is disclosed as an LP/other named investor for IGVCF, and Graphic coverage of the VCTF impact report identifies Injaro Ghana Venture Fund as one of the impactful funds anchored by VCTF.</t>
+        </is>
+      </c>
+    </row>
     <row r="98" ht="57" customHeight="1" s="16"/>
   </sheetData>
   <autoFilter ref="A1:O98"/>
@@ -34446,7 +34934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="16" min="1" max="1"/>
@@ -36209,7 +36697,7 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>VCTF is a Ghanaian quasi-government VC fund (not strictly a DFI)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
@@ -36267,7 +36755,7 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Venture Capital Trust Fund (VCTF) of Ghana</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -36679,15 +37167,70 @@
       <c r="I41" t="n">
         <v>0</v>
       </c>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
           <t>NSIA provided NGN 10bn anchor funding; FSD Africa supported facility set-up costs through technical assistance rather than a disclosed LP/co-investment commitment.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="45.75" customHeight="1" s="16"/>
+    <row r="42" ht="45.75" customHeight="1" s="16">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Oasis Africa VC Fund (OAF)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Oasis Capital Ghana</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2015/2016</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>50.5</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>PE / SME / VC</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Ghana + Cote d'Ivoire</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Venture Capital Trust Fund (VCTF)</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>3</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Dutch Good Growth Fund (DGGF); IFC; EIB</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Local investor base of five institutions and individuals at first close</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>VCTF government co-investment helped Oasis domicile the fund locally in Ghana. DGGF TA/legal work helped make the Ghana structure bankable for international DFIs; first close included DGGF, IFC and local investors, with EIB later disclosing an USD 8m commitment.</t>
+        </is>
+      </c>
+    </row>
     <row r="43" ht="45.75" customHeight="1" s="16"/>
     <row r="44" ht="57" customHeight="1" s="16"/>
     <row r="45" ht="45.75" customHeight="1" s="16"/>
@@ -36834,11 +37377,11 @@
         </is>
       </c>
       <c r="B7" s="23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Adenia Capital V; Africa50 Infrastructure Acceleration Fund (IAF); Ascent Rift Valley Fund II (ARVF II); Catalyst Fund II; Vantage Mezzanine IV (Pan-African sub-fund)</t>
+          <t>Adenia Capital V; Africa50 Infrastructure Acceleration Fund (IAF); Ascent Rift Valley Fund II (ARVF II); Catalyst Fund II; Vantage Mezzanine IV (Pan-African sub-fund); Oasis Africa VC Fund (OAF)</t>
         </is>
       </c>
       <c r="D7" s="23" t="inlineStr">
@@ -36859,11 +37402,11 @@
         </is>
       </c>
       <c r="B8" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>Adenia Capital V; Catalyst Fund II; Mediterrania Capital II / III / IV; Vantage Mezzanine IV (Pan-African sub-fund)</t>
+          <t>Adenia Capital V; Catalyst Fund II; Mediterrania Capital II / III / IV; Vantage Mezzanine IV (Pan-African sub-fund); Oasis Africa VC Fund (OAF)</t>
         </is>
       </c>
       <c r="D8" s="23" t="inlineStr">
@@ -37259,11 +37802,11 @@
         </is>
       </c>
       <c r="B24" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Africa Food Security Fund (AFSF)</t>
+          <t>Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Africa Food Security Fund (AFSF); Oasis Africa VC Fund (OAF)</t>
         </is>
       </c>
       <c r="D24" s="23" t="inlineStr">

</xml_diff>

<commit_message>
Add normalized asset focus approach taxonomy
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -26264,7 +26264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O97"/>
+  <dimension ref="A1:R97"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="16" min="1" max="1"/>
@@ -26359,6 +26359,21 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Asset class normalized</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Sector / thematic focus</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Investment approach</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="23.25" customHeight="1" s="16">
       <c r="A2" s="2" t="inlineStr">
@@ -26434,6 +26449,21 @@
           <t>PIC became 36th shareholder of Africa50 with USD 40m investment, signalling continental infrastructure commitment.</t>
         </is>
       </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="23.25" customHeight="1" s="16">
       <c r="A3" s="2" t="inlineStr">
@@ -26511,6 +26541,21 @@
           <t>PIC has been a recurring LP in Helios funds dating back to Helios II; specific commitment sizes not publicly disclosed.</t>
         </is>
       </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="16">
       <c r="A4" s="2" t="inlineStr">
@@ -26586,6 +26631,21 @@
           <t>PIC was an anchor LP at fund formation.</t>
         </is>
       </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="23.25" customHeight="1" s="16">
       <c r="A5" s="2" t="inlineStr">
@@ -26663,6 +26723,21 @@
           <t>PIC participated in Convergence Partners' digital infrastructure platform.</t>
         </is>
       </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Infrastructure; Digital / Technology</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="23.25" customHeight="1" s="16">
       <c r="A6" s="2" t="inlineStr">
@@ -26740,6 +26815,21 @@
           <t>Isibaya programme deploys to unlisted equity and infrastructure across SA and rest of Africa; PIC reports ~20% to alternatives overall.</t>
         </is>
       </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Infrastructure; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="23.25" customHeight="1" s="16">
       <c r="A7" s="2" t="inlineStr">
@@ -26817,6 +26907,21 @@
           <t>EPPF has been investing in PE for 10+ years; ~10% to alts total, ~4% to PE; selectively includes pan-Africa funds.</t>
         </is>
       </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Mixed / Multi-Asset</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="16">
       <c r="A8" s="2" t="inlineStr">
@@ -26892,6 +26997,21 @@
           <t>GEPF is ultimate asset owner; PIC executes.</t>
         </is>
       </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Infrastructure; Financial Inclusion / Financial Services</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Platform / Anchor Sponsor</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="23.25" customHeight="1" s="16">
       <c r="A9" s="2" t="inlineStr">
@@ -26967,6 +27087,21 @@
           <t>Latest committed fund LP investment; aligns with NIF sub-fund mandate.</t>
         </is>
       </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="23.25" customHeight="1" s="16">
       <c r="A10" s="2" t="inlineStr">
@@ -27044,6 +27179,21 @@
           <t>Federal Government injected USD 550m to scale energy infra; NIF is the direct-deal vehicle.</t>
         </is>
       </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Infrastructure; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="23.25" customHeight="1" s="16">
       <c r="A11" s="2" t="inlineStr">
@@ -27121,6 +27271,21 @@
           <t>Notable NIF direct PPP equity stake.</t>
         </is>
       </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="23.25" customHeight="1" s="16">
       <c r="A12" s="2" t="inlineStr">
@@ -27198,6 +27363,21 @@
           <t>NIF agribusiness anchor investment.</t>
         </is>
       </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Agriculture / Food Security</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="23.25" customHeight="1" s="16">
       <c r="A13" s="2" t="inlineStr">
@@ -27275,6 +27455,21 @@
           <t>NSIA has been an LP in Nigerian-focused PE funds; sizes not disclosed.</t>
         </is>
       </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="23.25" customHeight="1" s="16">
       <c r="A14" s="2" t="inlineStr">
@@ -27350,6 +27545,21 @@
           <t>Landmark first Nigerian-pension-funded infra fund.</t>
         </is>
       </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="34.5" customHeight="1" s="16">
       <c r="A15" s="2" t="inlineStr">
@@ -27427,6 +27637,21 @@
           <t>Largest PFA; alts are growing portion of portfolio under Multi-Fund Structure but per-fund sizes are not publicly disclosed.</t>
         </is>
       </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Infrastructure; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="23.25" customHeight="1" s="16">
       <c r="A16" s="2" t="inlineStr">
@@ -27504,6 +27729,21 @@
           <t>ARM Pension and ARM-Harith are part of the same group; intra-group LP commitments are an obvious starting point.</t>
         </is>
       </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="23.25" customHeight="1" s="16">
       <c r="A17" s="2" t="inlineStr">
@@ -27579,6 +27819,21 @@
           <t>Co-invested via Healthcare &amp; Pharma Subfund with B Investments and El-Ezaby Pharmacy.</t>
         </is>
       </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Co-investment</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="23.25" customHeight="1" s="16">
       <c r="A18" s="2" t="inlineStr">
@@ -27656,6 +27911,21 @@
           <t>Strategic healthcare platform co-developed with ADQ.</t>
         </is>
       </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Platform / Anchor Sponsor</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="23.25" customHeight="1" s="16">
       <c r="A19" s="2" t="inlineStr">
@@ -27733,6 +28003,21 @@
           <t>TSFE has been the on-ground co-investment vehicle for Gulf SWF deployment into Egypt across financial services, healthcare, infra.</t>
         </is>
       </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Infrastructure; Financial Inclusion / Financial Services; Healthcare; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Platform / Anchor Sponsor</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="23.25" customHeight="1" s="16">
       <c r="A20" s="2" t="inlineStr">
@@ -27810,6 +28095,21 @@
           <t>CDG Invest's direct-equity portfolio of Moroccan corporate stakes.</t>
         </is>
       </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Infrastructure; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="23.25" customHeight="1" s="16">
       <c r="A21" s="2" t="inlineStr">
@@ -27887,6 +28187,21 @@
           <t>CDG Invest manages CapMezzanine III, a mezzanine fund for Moroccan SMEs.</t>
         </is>
       </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="23.25" customHeight="1" s="16">
       <c r="A22" s="2" t="inlineStr">
@@ -27964,6 +28279,21 @@
           <t>CDG-managed infra investment vehicle.</t>
         </is>
       </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="23.25" customHeight="1" s="16">
       <c r="A23" s="2" t="inlineStr">
@@ -28041,6 +28371,21 @@
           <t>CDG has historically been an LP in Mediterrania PE funds focused on Maghreb mid-market.</t>
         </is>
       </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="23.25" customHeight="1" s="16">
       <c r="A24" s="2" t="inlineStr">
@@ -28116,6 +28461,21 @@
           <t>Joint investment with IFC and Fipar-Holding in retail/food platform.</t>
         </is>
       </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Agriculture / Food Security</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="23.25" customHeight="1" s="16">
       <c r="A25" s="2" t="inlineStr">
@@ -28193,6 +28553,21 @@
           <t>Ithmar describes Wessal as an investment vehicle / joint venture equally owned by five SWFs, not a conventional GP-managed fund. Named projects include Wessal Bouregreg and Wessal Casa-Port.</t>
         </is>
       </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Infrastructure; Real Estate / Housing</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Platform / Anchor Sponsor</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="23.25" customHeight="1" s="16">
       <c r="A26" s="2" t="inlineStr">
@@ -28270,6 +28645,21 @@
           <t>Newly-capitalised; intended as anchor for Moroccan sectoral funds.</t>
         </is>
       </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Mixed / Multi-Asset</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Platform / Anchor Sponsor</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="23.25" customHeight="1" s="16">
       <c r="A27" s="2" t="inlineStr">
@@ -28347,6 +28737,21 @@
           <t>GIPF Unlisted Investment Policy mandates ~10% PE + 5% RE; 307 underlying companies.</t>
         </is>
       </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Infrastructure; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="16">
       <c r="A28" s="2" t="inlineStr">
@@ -28424,6 +28829,21 @@
           <t>Stimulus is a flagship Namibian unlisted manager; GIPF is an anchor LP.</t>
         </is>
       </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="23.25" customHeight="1" s="16">
       <c r="A29" s="2" t="inlineStr">
@@ -28501,6 +28921,21 @@
           <t>Eos manages multiple unlisted funds anchored by GIPF.</t>
         </is>
       </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="23.25" customHeight="1" s="16">
       <c r="A30" s="2" t="inlineStr">
@@ -28574,6 +29009,21 @@
         </is>
       </c>
       <c r="O30" s="2" t="n"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="23.25" customHeight="1" s="16">
       <c r="A31" s="2" t="inlineStr">
@@ -28651,6 +29101,21 @@
           <t>Domestic housing facility — a developmental-investment direct programme.</t>
         </is>
       </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Infrastructure; Real Estate / Housing</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="23.25" customHeight="1" s="16">
       <c r="A32" s="2" t="inlineStr">
@@ -28726,6 +29191,21 @@
           <t>Part of BPOPF's domestic PE incubation programme.</t>
         </is>
       </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="23.25" customHeight="1" s="16">
       <c r="A33" s="2" t="inlineStr">
@@ -28801,6 +29281,21 @@
           <t>Part of BPOPF's incubation programme; anchor LP.</t>
         </is>
       </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="23.25" customHeight="1" s="16">
       <c r="A34" s="2" t="inlineStr">
@@ -28878,6 +29373,21 @@
           <t>Disclosed in industry sources; sizes not public.</t>
         </is>
       </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="23.25" customHeight="1" s="16">
       <c r="A35" s="2" t="inlineStr">
@@ -28955,6 +29465,21 @@
           <t>BPOPF targets ~10% in alternatives including PE, infra, RE.</t>
         </is>
       </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Infrastructure; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="23.25" customHeight="1" s="16">
       <c r="A36" s="2" t="inlineStr">
@@ -29030,6 +29555,21 @@
           <t>NSSF Uganda was a founding LP alongside EU and IFAD; fund now at EUR 20m total commitments. [CORRECTED in Phase 6: NSSF Uganda's actual founding ticket was EUR 2m, alongside EUR 10m from EU/IFAD, for the EUR 12m total first close. Fund subsequently grew to EUR 20m via FCA Investments + Soros Economic Development Fund.]</t>
         </is>
       </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Agriculture / Food Security</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="23.25" customHeight="1" s="16">
       <c r="A37" s="2" t="inlineStr">
@@ -29107,6 +29647,21 @@
           <t>NSSF Uganda discloses ~20% alts; real estate dominant historically, infra/PE growing.</t>
         </is>
       </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Infrastructure; Real Estate / Housing; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="23.25" customHeight="1" s="16">
       <c r="A38" s="2" t="inlineStr">
@@ -29182,6 +29737,21 @@
           <t>Reported among Catalyst II's LPs.</t>
         </is>
       </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="23.25" customHeight="1" s="16">
       <c r="A39" s="2" t="inlineStr">
@@ -29257,6 +29827,21 @@
           <t>Joint pan-African infra fund with Gemcorp.</t>
         </is>
       </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Platform / Holding Company</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Platform / Anchor Sponsor</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="23.25" customHeight="1" s="16">
       <c r="A40" s="2" t="inlineStr">
@@ -29332,6 +29917,21 @@
           <t>Multi-party rail-and-port infrastructure development.</t>
         </is>
       </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="23.25" customHeight="1" s="16">
       <c r="A41" s="2" t="inlineStr">
@@ -29409,6 +30009,21 @@
           <t>FSDEA portfolio includes PE funds among other asset classes; per-fund detail not publicly disclosed.</t>
         </is>
       </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Mixed / Multi-Asset</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Infrastructure; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="23.25" customHeight="1" s="16">
       <c r="A42" s="2" t="inlineStr">
@@ -29484,6 +30099,21 @@
           <t>FONSIS and KfW/World Bank launched Oyass Capital as an SME-focused private-equity fund/financing vehicle; FONSIS says SEAF received the management mandate after an international tender.</t>
         </is>
       </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>SME Finance; Financial Inclusion / Financial Services</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Platform / Anchor Sponsor</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="23.25" customHeight="1" s="16">
       <c r="A43" s="2" t="inlineStr">
@@ -29561,6 +30191,21 @@
           <t>FONSIS's primary mandate is direct strategic investment in Senegalese transformational projects.</t>
         </is>
       </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Infrastructure; Agriculture / Food Security; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="23.25" customHeight="1" s="16">
       <c r="A44" s="2" t="inlineStr">
@@ -29638,6 +30283,21 @@
           <t>AgDF holds equity in selected Rwandan strategic companies.</t>
         </is>
       </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="23.25" customHeight="1" s="16">
       <c r="A45" s="2" t="inlineStr">
@@ -29715,6 +30375,21 @@
           <t>RSSB holds significant direct equity in Rwandan strategic enterprises.</t>
         </is>
       </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="16">
       <c r="A46" s="2" t="inlineStr">
@@ -29790,6 +30465,21 @@
           <t>34% of portfolio in alts as of 2023; 2024 strategy shift to rebalance toward fixed income announced.</t>
         </is>
       </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Infrastructure; Real Estate / Housing; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="23.25" customHeight="1" s="16">
       <c r="A47" s="2" t="inlineStr">
@@ -29867,6 +30557,21 @@
           <t>Significant historic direct-equity holdings in listed and unlisted Ghanaian firms.</t>
         </is>
       </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Agriculture / Food Security; Financial Inclusion / Financial Services; Real Estate / Housing</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="23.25" customHeight="1" s="16">
       <c r="A48" s="2" t="inlineStr">
@@ -29944,6 +30649,21 @@
           <t>Domestic infrastructure direct-deal mandate.</t>
         </is>
       </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Infrastructure; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="23.25" customHeight="1" s="16">
       <c r="A49" s="2" t="inlineStr">
@@ -30021,6 +30741,21 @@
           <t>FGIS has built equity stakes in Gabonese banking and infrastructure.</t>
         </is>
       </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Infrastructure; Financial Inclusion / Financial Services; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="23.25" customHeight="1" s="16">
       <c r="A50" s="2" t="inlineStr">
@@ -30098,6 +30833,21 @@
           <t>Mandate includes strategic co-investments.</t>
         </is>
       </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Infrastructure; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Platform / Anchor Sponsor</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="16">
       <c r="A51" s="2" t="inlineStr">
@@ -30173,6 +30923,21 @@
           <t>First disclosed Ghanaian pension trustee commitment to SME debt under Ghana's new 5% alternative-assets rule. Co-committed alongside Norfund (USD 15m); GIP capital base raised to ~USD 70m.</t>
         </is>
       </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Co-investment</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="16">
       <c r="A52" s="2" t="inlineStr">
@@ -30248,6 +31013,21 @@
           <t>Ghanaian pension capital is &gt;2/3 of Ci Gaba's first-close commitments. West Africa's first domestically-domiciled private fund of funds; target size GHS 1bn / USD 91m.</t>
         </is>
       </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Fund of Funds</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Fund of Funds LP</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="34.5" customHeight="1" s="16">
       <c r="A53" s="2" t="inlineStr">
@@ -30323,6 +31103,21 @@
           <t>One of Ghana's largest private trustees; LP alongside AXIS, Stanbic IMS, CAL Asset Management, FSDAi, Small Foundation, FMO.</t>
         </is>
       </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Fund of Funds</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Fund of Funds LP</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="23.25" customHeight="1" s="16">
       <c r="A54" s="2" t="inlineStr">
@@ -30398,6 +31193,21 @@
           <t>Separate from the 2025 PIC-Africa50 commitment. PIC's largest disclosed pan-African institutional equity position.</t>
         </is>
       </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="23.25" customHeight="1" s="16">
       <c r="A55" s="2" t="inlineStr">
@@ -30475,6 +31285,21 @@
           <t>First Indian Ocean shareholder of AFC; joined with Sierra Leone and GIIF Ghana.</t>
         </is>
       </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="23.25" customHeight="1" s="16">
       <c r="A56" s="2" t="inlineStr">
@@ -30552,6 +31377,21 @@
           <t>GIIF deploys its own balance sheet into AFC; aligns with GIIF's domestic-infra mandate.</t>
         </is>
       </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="34.5" customHeight="1" s="16">
       <c r="A57" s="2" t="inlineStr">
@@ -30629,6 +31469,21 @@
           <t>Mauritius participates via NPF and NSF jointly.</t>
         </is>
       </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="34.5" customHeight="1" s="16">
       <c r="A58" s="2" t="inlineStr">
@@ -30706,6 +31561,21 @@
           <t>Joint Mauritian participation alongside NPF.</t>
         </is>
       </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="23.25" customHeight="1" s="16">
       <c r="A59" s="2" t="inlineStr">
@@ -30783,6 +31653,21 @@
           <t>First Central African pension fund to take AFC equity. Important precedent for CIPRES-supervised funds.</t>
         </is>
       </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="34.5" customHeight="1" s="16">
       <c r="A60" s="2" t="inlineStr">
@@ -30860,6 +31745,21 @@
           <t>Distinct from CNSS Gabon and FGIS. NEW entity vs Phase 1 roster — should be added to Pension Funds tab.</t>
         </is>
       </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="23.25" customHeight="1" s="16">
       <c r="A61" s="2" t="inlineStr">
@@ -30937,6 +31837,21 @@
           <t>Ivorian sovereign equity participation.</t>
         </is>
       </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="23.25" customHeight="1" s="16">
       <c r="A62" s="2" t="inlineStr">
@@ -31010,6 +31925,21 @@
         </is>
       </c>
       <c r="O62" s="2" t="n"/>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="23.25" customHeight="1" s="16">
       <c r="A63" s="2" t="inlineStr">
@@ -31085,6 +32015,21 @@
           <t>First North African shareholder of AFC; widens TSFE-NOSI Egypt's institutional alts footprint outside the country.</t>
         </is>
       </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="23.25" customHeight="1" s="16">
       <c r="A64" s="2" t="inlineStr">
@@ -31160,6 +32105,21 @@
           <t>Distinct from FONSIS; Senegal's civil-service deposit institution. Africa50-IAF was named 'African first' as it was majority African-LP funded.</t>
         </is>
       </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="23.25" customHeight="1" s="16">
       <c r="A65" s="2" t="inlineStr">
@@ -31235,6 +32195,21 @@
           <t>Beninese deposit-and-investment institution joining Africa50-IAF.</t>
         </is>
       </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="23.25" customHeight="1" s="16">
       <c r="A66" s="2" t="inlineStr">
@@ -31310,6 +32285,21 @@
           <t>First disclosed CIPRES-zone pension fund LP commitment to a pan-African PE-style infrastructure fund.</t>
         </is>
       </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="23.25" customHeight="1" s="16">
       <c r="A67" s="2" t="inlineStr">
@@ -31385,6 +32375,21 @@
           <t>CDG Invest is the asset-management subsidiary of CDG Morocco.</t>
         </is>
       </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="23.25" customHeight="1" s="16">
       <c r="A68" s="2" t="inlineStr">
@@ -31460,6 +32465,21 @@
           <t>CBK Pension Fund (Central Bank of Kenya staff pension) committed alongside Norfund and IFU. CBK PF remained LP through subsequent closes.</t>
         </is>
       </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>Financial Inclusion / Financial Services</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="23.25" customHeight="1" s="16">
       <c r="A69" s="2" t="inlineStr">
@@ -31535,6 +32555,21 @@
           <t>NAPSA is the third anchor alongside BII (USD 37.5m) and Swedfund (USD 15m); GIP Zambia plans to deploy USD 300m over 15 years to ~150 Zambian SMEs in local currency. Largest single disclosed Zambian-pension alts commitment.</t>
         </is>
       </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="23.25" customHeight="1" s="16">
       <c r="A70" s="2" t="inlineStr">
@@ -31610,6 +32645,21 @@
           <t>Adenia Capital V LP roster includes 'Kenyan pension funds' but no specific funds named at close-disclosure level. Likely candidates: schemes that participate via KEPFIC consortium.</t>
         </is>
       </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="23.25" customHeight="1" s="16">
       <c r="A71" s="2" t="inlineStr">
@@ -31685,6 +32735,21 @@
           <t>Adenia Capital V LP roster includes 'Ghanaian pension funds' but no specific trustees named at close-disclosure level.</t>
         </is>
       </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="23.25" customHeight="1" s="16">
       <c r="A72" s="2" t="inlineStr">
@@ -31760,6 +32825,21 @@
           <t>Specifically named as LP in Adenia V's hard-cap close; PIC commitment size not disclosed.</t>
         </is>
       </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="23.25" customHeight="1" s="16">
       <c r="A73" s="2" t="inlineStr">
@@ -31837,6 +32917,21 @@
           <t>Catalyst Fund II disclosed 'local pension funds and family offices' as LPs alongside CDC/BII USD 30m, EIB, IFC, Proparco, Swedfund. NSSF Uganda is known to have committed (per earlier industry reporting); other names not publicly disclosed.</t>
         </is>
       </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="23.25" customHeight="1" s="16">
       <c r="A74" s="2" t="inlineStr">
@@ -31914,6 +33009,21 @@
           <t>Retained as an aggregate consortium archetype only. IFC reports KEPFIC mobilized $113m into two housing projects and facilitated two member-fund investments, with a road infrastructure bond near closing. Individual KEPFIC member-only rows removed because membership alone is not allocator-to-vehicle commitment evidence.</t>
         </is>
       </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>Infrastructure; Real Estate / Housing; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="23.25" customHeight="1" s="16">
       <c r="A75" s="2" t="inlineStr">
@@ -31989,6 +33099,21 @@
           <t>Historical first: described as 'the first pension fund in East African private equity'. ARVF I total first close USD 50m.</t>
         </is>
       </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="23.25" customHeight="1" s="16">
       <c r="A76" s="2" t="inlineStr">
@@ -32064,6 +33189,21 @@
           <t>Commitment made via STANLIB Kenya as fund manager. Trustee Wallace Kantai: 'first of many investments of this kind by our fund'.</t>
         </is>
       </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="23.25" customHeight="1" s="16">
       <c r="A77" s="2" t="inlineStr">
@@ -32141,6 +33281,21 @@
           <t>Source notes 'three pension funds (two from Kenya Power Pension Fund and one from Nation Media Group Staff Pension Fund)'. Two KPLC PF commitments likely reflect the KPLC main scheme + KPLC Staff Retirement Benefits Scheme separately.</t>
         </is>
       </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="34.5" customHeight="1" s="16">
       <c r="A78" s="2" t="inlineStr">
@@ -32218,6 +33373,21 @@
           <t>Re-up after ARVF I; NMG remains an LP.</t>
         </is>
       </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="45.75" customHeight="1" s="16">
       <c r="A79" s="2" t="inlineStr">
@@ -32293,6 +33463,21 @@
           <t>NSIA was an LP alongside AfDB, CDC Group/BII, and Dutch Good Growth Fund (DGGF) in Sahel's FAFIN. NSIA's earliest disclosed PE fund LP position alongside DFIs.</t>
         </is>
       </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>Agriculture / Food Security</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="23.25" customHeight="1" s="16">
       <c r="A80" s="2" t="inlineStr">
@@ -32370,6 +33555,21 @@
           <t>ACA historically championed PE inclusion as allowable Nigerian pension asset class. Some PFA commitments to CAPE funds confirmed by ACA's stated 'institutional investor base, primarily pension funds and DFIs'; specific PFA names not individually disclosed.</t>
         </is>
       </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="34.5" customHeight="1" s="16">
       <c r="A81" s="2" t="inlineStr">
@@ -32445,6 +33645,21 @@
           <t>Three regional firsts per RSSB CEO Regis Rugemanshuro: (i) FIRST public pension-fund-led initiative focused exclusively on SME financing; (ii) FIRST permanent capital vehicle anchored by a pension fund; (iii) FIRST pension fund dedicating a TA facility in a fund. Fund target USD 100m. Enko Capital parent has USD 1.6bn AUM. FSDA structured the deal + potential guarantee facility.</t>
         </is>
       </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="23.25" customHeight="1" s="16">
       <c r="A82" s="2" t="inlineStr">
@@ -32522,6 +33737,21 @@
           <t>Retained as an aggregate consortium archetype only. Public sources report actual collective AOFSA member commitments; individual member-only rows removed because the public evidence does not allocate the commitments by named member fund.</t>
         </is>
       </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>Infrastructure; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="23.25" customHeight="1" s="16">
       <c r="A83" s="2" t="inlineStr">
@@ -32597,6 +33827,21 @@
           <t>Second Ghana fund anchored solely by local investors (after Injaro IGVCF). Petra Trust named alongside Axis Pensions, VCTF, and CAMCOL schemes. Mirepa fund focuses on light manufacturing, technology, cleantech, agribusiness, healthcare, financial services.</t>
         </is>
       </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>SME Finance; Agriculture / Food Security; Financial Inclusion / Financial Services; Healthcare; Climate / Energy Transition; Digital / Technology</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="45.75" customHeight="1" s="16">
       <c r="A84" s="2" t="inlineStr">
@@ -32672,6 +33917,21 @@
           <t>Axis Pensions named LP alongside Petra Trust, VCTF, CAMCOL schemes. Predates Axis's later commitments to GIP Ghana (Apr 2026) and Ci-Gaba FoF (Mar 2026).</t>
         </is>
       </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="90.75" customHeight="1" s="16">
       <c r="A85" s="2" t="inlineStr">
@@ -32747,6 +34007,21 @@
           <t>CAL Asset Management Company Limited (CAMCOL) is one of the major Ghanaian pension asset managers. Underlying pension scheme identities not individually disclosed.</t>
         </is>
       </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="34.5" customHeight="1" s="16">
       <c r="A86" s="2" t="inlineStr">
@@ -32822,6 +34097,21 @@
           <t>FIRST Ghana fund of its kind anchored by local pension funds (per Injaro press release). Predates Mirepa I (2023) and Ci-Gaba (2026). Specific Ghanaian pension fund names not disclosed in public sources but precedent-setting.</t>
         </is>
       </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="34.5" customHeight="1" s="16">
       <c r="A87" t="inlineStr">
@@ -32897,6 +34187,21 @@
           <t>DGGF names PIC on behalf of GEPF among first-round AFSF investors alongside AfDB, CDC Group/BII, DGGF, IFU, and EBID; Kuramo later joined, bringing fund commitments to USD 84m.</t>
         </is>
       </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>Agriculture / Food Security</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="45.75" customHeight="1" s="16">
       <c r="A88" t="inlineStr">
@@ -32974,6 +34279,21 @@
           <t>NSIA names Alitheia IDF among investments supporting women-led and women-impacting businesses. Specific NSIA ticket size not publicly disclosed.</t>
         </is>
       </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>Infrastructure; Gender Lens</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="34.5" customHeight="1" s="16">
       <c r="A89" t="inlineStr">
@@ -33051,6 +34371,21 @@
           <t>NSIA names Ingressive Capital among investments supporting women-led and women-impacting businesses. Public NSIA source does not identify a specific vintage, so retained as platform/fund exposure.</t>
         </is>
       </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>Infrastructure; SME Finance; Digital / Technology</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="34.5" customHeight="1" s="16">
       <c r="A90" t="inlineStr">
@@ -33126,6 +34461,21 @@
           <t>NSIA impact report states the Authority invested USD 5m in Verod Growth Fund II in 2017.</t>
         </is>
       </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="23.25" customHeight="1" s="16">
       <c r="A91" t="inlineStr">
@@ -33203,6 +34553,21 @@
           <t>NSIA impact report states the Authority subsequently invested in Verod Growth Fund III, with 8% of the USD 7.5m commitment disbursed at the time of reporting.</t>
         </is>
       </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="23.25" customHeight="1" s="16">
       <c r="A92" t="inlineStr">
@@ -33278,6 +34643,21 @@
           <t>IFC and NSIA partnered to finance MedServe, NSIA's wholly owned healthcare subsidiary, to scale diagnostic centers, cancer care facilities and cath labs across Nigerian states.</t>
         </is>
       </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>Direct Investment</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="124.5" customHeight="1" s="16">
       <c r="A93" t="inlineStr">
@@ -33355,6 +34735,21 @@
           <t>InfraCredit is a specialised infrastructure credit enhancement facility established by NSIA with GuarantCo/PIDG. NSIA FY2025 statements report a 43.88% retained ownership interest after shareholder changes.</t>
         </is>
       </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>Guarantee / Credit Enhancement</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>Guarantee-backed Instrument</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="124.5" customHeight="1" s="16">
       <c r="A94" t="inlineStr">
@@ -33430,6 +34825,21 @@
           <t>NSIA invested NGN 10bn into a multi-funder revolving construction finance facility developed with InfraCredit to support greenfield infrastructure projects backed by InfraCredit guarantees.</t>
         </is>
       </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>Guarantee / Credit Enhancement</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>Infrastructure; Climate / Energy Transition</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>Guarantee-backed Instrument</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="79.5" customHeight="1" s="16">
       <c r="A95" t="inlineStr">
@@ -33507,6 +34917,21 @@
           <t>VCTF 2015 annual report states VCTF made a USD 2m commitment to Oasis Africa Fund Limited, Oasis Capital Partners second fund. DGGF later described OAF as Ghana-domiciled to access VCTF government co-investment and noted the structure helped crowd in international DFIs.</t>
         </is>
       </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>Infrastructure; SME Finance</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="34.5" customHeight="1" s="16">
       <c r="A96" t="inlineStr">
@@ -33582,6 +35007,21 @@
           <t>VCTF is named in the Mirepa LP group alongside Petra Trust, Axis Pensions and CAMCOL-managed pension schemes; public coverage describes VCTF as leading the investment.</t>
         </is>
       </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="45.75" customHeight="1" s="16">
       <c r="A97" t="inlineStr">
@@ -33655,6 +35095,21 @@
       <c r="O97" t="inlineStr">
         <is>
           <t>VCTF is disclosed as an LP/other named investor for IGVCF, and Graphic coverage of the VCTF impact report identifies Injaro Ghana Venture Fund as one of the impactful funds anchored by VCTF.</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>Infrastructure; SME Finance</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
         </is>
       </c>
     </row>
@@ -33683,7 +35138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:S15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="16" min="1" max="1"/>
@@ -33785,6 +35240,21 @@
           <t>Source URL</t>
         </is>
       </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Asset class normalized</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Sector / thematic focus</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Investment approach</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="26" t="inlineStr">
@@ -33865,6 +35335,21 @@
           <t>https://archive.fsdafrica.org/arm-harith-and-fsd-africa-investments-announce-gbp-10m-commitment-to-unlock-nigerian-pension-funds-and-catalyse-local-capital-for-infrastructure/</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Infrastructure; Climate / Energy Transition</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="26" t="inlineStr">
@@ -33947,6 +35432,21 @@
           <t>https://www.ecofinagency.com/news-finances/2502-53253-nigerian-investment-firm-sahel-capital-launches-55-million-fund-to-narrow-farm-finance-gap</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Agriculture / Food Security</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
@@ -34023,6 +35523,21 @@
         </is>
       </c>
       <c r="P4" s="26" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Fund of Funds</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="26" t="inlineStr">
@@ -34101,6 +35616,21 @@
         </is>
       </c>
       <c r="P5" s="26" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Infrastructure; Climate / Energy Transition</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -34183,6 +35713,21 @@
           <t>https://www.ifc.org/en/stories/2023/pooling-pensions-in-kenya</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Infrastructure; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="26" t="inlineStr">
@@ -34265,6 +35810,21 @@
           <t>https://www.ifc.org/en/stories/2023/pooling-pensions-in-kenya</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Infrastructure; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="26" t="inlineStr">
@@ -34347,6 +35907,21 @@
           <t>https://www.ifc.org/en/stories/2023/pooling-pensions-in-kenya</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="26" t="inlineStr">
@@ -34429,6 +36004,21 @@
           <t>https://www.ifc.org/en/stories/2023/pooling-pensions-in-kenya</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="26" t="inlineStr">
@@ -34511,6 +36101,21 @@
           <t>https://www.engineeringnews.co.za/article/aofsa-exceeds-infrastructure-investment-target-as-it-marks-first-anniversary-2022-11-21</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="26" t="inlineStr">
@@ -34593,6 +36198,21 @@
           <t>https://www.engineeringnews.co.za/article/aofsa-exceeds-infrastructure-investment-target-as-it-marks-first-anniversary-2022-11-21</t>
         </is>
       </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="26" t="inlineStr">
@@ -34675,6 +36295,21 @@
           <t>https://www.engineeringnews.co.za/article/aofsa-exceeds-infrastructure-investment-target-as-it-marks-first-anniversary-2022-11-21</t>
         </is>
       </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="26" t="inlineStr">
@@ -34757,6 +36392,21 @@
           <t>https://www.engineeringnews.co.za/article/aofsa-exceeds-infrastructure-investment-target-as-it-marks-first-anniversary-2022-11-21</t>
         </is>
       </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -34839,6 +36489,21 @@
           <t>https://www.ifc.org/en/stories/2023/pooling-pensions-in-kenya ; https://www.midaadvisors.com/advisory-firm-financing-the-development-of-critical-infrastructure-in-kenya-with-local-institutional-capital</t>
         </is>
       </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Infrastructure; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -34919,6 +36584,21 @@
       <c r="P15" t="inlineStr">
         <is>
           <t>https://www.engineeringnews.co.za/article/aofsa-exceeds-infrastructure-investment-target-as-it-marks-first-anniversary-2022-11-21 ; https://www.midaadvisors.com/advisory-firm-what-we-do/institutional-investors-capacity-development</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Infrastructure; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Mandate / Pipeline Only</t>
         </is>
       </c>
     </row>
@@ -34934,7 +36614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:O42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="16" min="1" max="1"/>
@@ -35019,6 +36699,21 @@
           <t>Co-investor pattern note</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Asset class normalized</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Sector / thematic focus</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Investment approach</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="34.5" customHeight="1" s="16">
       <c r="A4" s="2" t="inlineStr">
@@ -35077,6 +36772,21 @@
           <t>BII-anchored DFI + 1 Ghanaian pension trustee. First Ghanaian PF commitment under 5% alts rule.</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="23.25" customHeight="1" s="16">
       <c r="A5" s="2" t="inlineStr">
@@ -35133,6 +36843,21 @@
           <t>Largest single disclosed Zambian-pension alts commitment. Trilateral DFI+pension anchor model.</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="23.25" customHeight="1" s="16">
       <c r="A6" s="2" t="inlineStr">
@@ -35193,6 +36918,21 @@
           <t>West Africa's first domestically-domiciled private FoF. Ghanaian pensions &gt;2/3 of first close.</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Fund of Funds</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Fund of Funds LP</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="23.25" customHeight="1" s="16">
       <c r="A7" s="2" t="inlineStr">
@@ -35253,6 +36993,21 @@
           <t>Landmark first-Nigerian-pension-funded infra fund.</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="34.5" customHeight="1" s="16">
       <c r="A8" s="2" t="inlineStr">
@@ -35311,6 +37066,21 @@
           <t>FONSIS source describes Oyass Capital as an SME-focused private-equity fund/financing vehicle set up with KfW/World Bank support; management mandate awarded to SEAF.</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Infrastructure; SME Finance; Financial Inclusion / Financial Services</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="23.25" customHeight="1" s="16">
       <c r="A9" s="2" t="inlineStr">
@@ -35369,6 +37139,21 @@
           <t>NSSF Uganda founding LP alongside EU + IFAD. [Phase 6 correction: NSSF Uganda's founding contribution was EUR 2m (not EUR 12m); EUR 12m was the TOTAL first close including EU/IFAD EUR 10m. Later EUR 8m added by Soros Economic Development Fund + FCA Investments brought total to EUR 20m.]</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Agriculture / Food Security</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="34.5" customHeight="1" s="16">
       <c r="A10" s="2" t="inlineStr">
@@ -35425,6 +37210,21 @@
           <t>Historical pioneer fund for East African pension PE participation.</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="23.25" customHeight="1" s="16">
       <c r="A11" s="2" t="inlineStr">
@@ -35485,6 +37285,21 @@
           <t>Strong DFI cluster alongside re-up of East African pension LPs. Source narrative: ARVF was 'the only local PE fund continually unlocking local pension investment' as of 2015.</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="34.5" customHeight="1" s="16">
       <c r="A12" s="2" t="inlineStr">
@@ -35541,6 +37356,21 @@
           <t>~30 LPs total; &gt;60% historical DFI re-ups; categorical 'Kenyan + Ghanaian pension funds' mentioned in press release but not individually named. [Phase 6 update: comprehensive LP list confirmed via EIB disclosure. 10 DFIs + PIC SA + categorical Kenyan/Ghanaian PFs + family offices = ~30 LP entities total.]</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="34.5" customHeight="1" s="16">
       <c r="A13" s="2" t="inlineStr">
@@ -35597,6 +37427,21 @@
           <t>Single largest East African PE fund with disclosed local-pension cohort.</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="23.25" customHeight="1" s="16">
       <c r="A14" s="2" t="inlineStr">
@@ -35657,6 +37502,21 @@
           <t>PIC has been recurring LP since Helios II; sizes not publicly disclosed.</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="23.25" customHeight="1" s="16">
       <c r="A15" s="2" t="inlineStr">
@@ -35715,6 +37575,21 @@
           <t>Vantage's 'historical pattern' of substantial SA pension LP base; specific names not publicly itemised.</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="23.25" customHeight="1" s="16">
       <c r="A16" s="2" t="inlineStr">
@@ -35775,6 +37650,21 @@
           <t>Maghreb-focused; CDG Morocco historical LP.</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="34.5" customHeight="1" s="16">
       <c r="A17" s="2" t="inlineStr">
@@ -35833,6 +37723,21 @@
           <t>Evergreen platform; CBK Pension Fund Kenya was first African pension LP in 2018; multiple closes since.</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Platform / Holding Company</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Financial Inclusion / Financial Services; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="16">
       <c r="A18" s="2" t="inlineStr">
@@ -35889,6 +37794,21 @@
           <t>BPOPF domestic incubation programme — single-LP-anchor model.</t>
         </is>
       </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="23.25" customHeight="1" s="16">
       <c r="A19" s="2" t="inlineStr">
@@ -35945,6 +37865,21 @@
           <t>Sister vehicle to Aleyo; BPOPF anchor.</t>
         </is>
       </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="23.25" customHeight="1" s="16">
       <c r="A20" s="2" t="inlineStr">
@@ -36005,6 +37940,21 @@
           <t>Continental infrastructure platform. PIC's 2025 commitment is largest single PF equity shareholding.</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="23.25" customHeight="1" s="16">
       <c r="A21" s="2" t="inlineStr">
@@ -36063,6 +38013,21 @@
           <t>First major pan-African infra fund MAJORITY-funded by African institutions. Africa50's flagship LP-style vehicle.</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="23.25" customHeight="1" s="16">
       <c r="A22" s="2" t="inlineStr">
@@ -36125,6 +38090,21 @@
           <t>Continental institutional-equity vehicle. By count of institutions, AFC participation is the MOST COMMON form of cross-border African pension/SWF alts deployment.</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="16">
       <c r="A23" s="2" t="inlineStr">
@@ -36183,6 +38163,21 @@
           <t>PIC anchor; significant African-LP-funded infra fund.</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="23.25" customHeight="1" s="16">
       <c r="A24" s="2" t="inlineStr">
@@ -36243,6 +38238,21 @@
           <t>Digital infrastructure; PIC participant.</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Infrastructure; Digital / Technology</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="34.5" customHeight="1" s="16">
       <c r="A25" s="2" t="inlineStr">
@@ -36301,6 +38311,21 @@
           <t>Ithmar describes Wessal as a joint investment vehicle, equally owned by five SWFs. Specific launched projects: Wessal Bouregreg and Wessal Casa-Port.</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Infrastructure; Real Estate / Housing</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="23.25" customHeight="1" s="16">
       <c r="A26" s="2" t="inlineStr">
@@ -36357,6 +38382,21 @@
           <t>Capitalised Moroccan strategic SWF — anchor for sub-funds.</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Mixed / Multi-Asset</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Multi-Sector</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="16">
       <c r="A27" s="2" t="inlineStr">
@@ -36417,6 +38457,21 @@
           <t>NIF is NSIA's direct-deal sub-fund; received USD 550m additional govt funding FY24.</t>
         </is>
       </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Infrastructure; Agriculture / Food Security; Healthcare</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="23.25" customHeight="1" s="16">
       <c r="A28" s="2" t="inlineStr">
@@ -36475,6 +38530,21 @@
           <t>Bilateral SWF healthcare platform.</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Platform / Anchor Sponsor</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="45.75" customHeight="1" s="16">
       <c r="A29" s="2" t="inlineStr">
@@ -36529,6 +38599,21 @@
           <t>NSIA's earliest disclosed PE fund LP position; alongside three DFIs.</t>
         </is>
       </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Agriculture / Food Security</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="90.75" customHeight="1" s="16">
       <c r="A30" s="2" t="inlineStr">
@@ -36591,6 +38676,21 @@
           <t>First Nigerian PE firm (founded 1997); CAPE I was Nigeria's first PE fund (1998). Continental pioneer of pension-PE inclusion.</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="23.25" customHeight="1" s="16">
       <c r="A31" s="2" t="inlineStr">
@@ -36647,6 +38747,21 @@
           <t>First permanent capital vehicle anchored by an African pension fund (per RSSB CEO). Three regional firsts: pension-fund-led SME-only mandate, anchor permanent-capital vehicle, pension-fund TA facility.</t>
         </is>
       </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="23.25" customHeight="1" s="16">
       <c r="A32" s="2" t="inlineStr">
@@ -36705,6 +38820,21 @@
           <t>Second Ghana fund anchored solely by local investors (after Injaro IGVCF). 100% local-LP-funded. Confirms Ghana's emerging mandated-minimum-alts policy is producing real deal flow.</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="23.25" customHeight="1" s="16">
       <c r="A33" s="2" t="inlineStr">
@@ -36763,6 +38893,21 @@
           <t>FIRST Ghana fund of its kind anchored by local pension funds. Historical precedent for Mirepa I, Ci-Gaba, GIP Ghana model. Ghana cedi-denominated.</t>
         </is>
       </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>SME Finance</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="23.25" customHeight="1" s="16">
       <c r="A34" t="inlineStr">
@@ -36817,6 +38962,21 @@
           <t>DGGF news release names PIC/GEPF in first-round investor group alongside DFIs and DGGF; Kuramo subsequently joined to bring commitments to USD 84m.</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Agriculture / Food Security</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="23.25" customHeight="1" s="16">
       <c r="A35" t="inlineStr">
@@ -36870,6 +39030,21 @@
           <t>NSIA names Alitheia IDF as an investment; SEDF describes Alitheia IDF as a USD 100m gender-lens fund. NSIA ticket size not disclosed.</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Gender Lens</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="16">
       <c r="A36" t="inlineStr">
@@ -36918,6 +39093,21 @@
           <t>NSIA names Ingressive Capital as an investment; specific NSIA vehicle/vintage and ticket size not publicly disclosed.</t>
         </is>
       </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>SME Finance; Digital / Technology</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="34.5" customHeight="1" s="16">
       <c r="A37" t="inlineStr">
@@ -36964,6 +39154,21 @@
           <t>NSIA impact report identifies a USD 5m FGF commitment to Verod Growth Fund II.</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="23.25" customHeight="1" s="16">
       <c r="A38" t="inlineStr">
@@ -37012,6 +39217,21 @@
           <t>NSIA impact report identifies a USD 7.5m FGF commitment to Verod Growth Fund III.</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="34.5" customHeight="1" s="16">
       <c r="A39" t="inlineStr">
@@ -37068,6 +39288,21 @@
           <t>IFC provided roughly NGN 14.2bn / USD 24.5m local-currency financing for NSIA's wholly owned MedServe expansion program.</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Direct Equity / Strategic Stake</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="34.5" customHeight="1" s="16">
       <c r="A40" t="inlineStr">
@@ -37126,6 +39361,21 @@
           <t>NSIA established InfraCredit with GuarantCo/PIDG. Later shareholders/backers include KfW, AfDB, InfraCo Africa, AFC, insurers, and Nigerian pension shareholders.</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Guarantee / Credit Enhancement</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Guarantee-backed Instrument</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="16">
       <c r="A41" t="inlineStr">
@@ -37172,6 +39422,21 @@
           <t>NSIA provided NGN 10bn anchor funding; FSD Africa supported facility set-up costs through technical assistance rather than a disclosed LP/co-investment commitment.</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Guarantee / Credit Enhancement</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Infrastructure; Digital / Technology</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Guarantee-backed Instrument</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="45.75" customHeight="1" s="16">
       <c r="A42" t="inlineStr">
@@ -37228,6 +39493,21 @@
       <c r="L42" t="inlineStr">
         <is>
           <t>VCTF government co-investment helped Oasis domicile the fund locally in Ghana. DGGF TA/legal work helped make the Ghana structure bankable for international DFIs; first close included DGGF, IFC and local investors, with EIB later disclosing an USD 8m commitment.</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>SME Finance; Financial Inclusion / Financial Services</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Virunga Africa Fund I RSSB commitment
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -4908,7 +4908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F199"/>
+  <dimension ref="A1:F200"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="16" min="1" max="2"/>
@@ -11283,6 +11283,38 @@
       <c r="F199" t="inlineStr">
         <is>
           <t>VCTF mandate as government-backed venture capital fund of funds focused on SME venture funds</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>RSSB Rwanda</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Fund launch / press release</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Kigali International Financial Centre establishes a $250M pan-African Virunga Africa Fund I</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>June 2026</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>https://www.rssb.rw/fileadmin/user_upload/Kigali_International_Financial_Centre.pdf</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Virunga Africa Fund I launch; QIA and RSSB named as anchor/cornerstone investors; Admaius manager; USD 250m fund size and pan-African sector focus</t>
         </is>
       </c>
     </row>
@@ -26264,7 +26296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R97"/>
+  <dimension ref="A1:R98"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="16" min="1" max="1"/>
@@ -35113,7 +35145,96 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="57" customHeight="1" s="16"/>
+    <row r="98" ht="57" customHeight="1" s="16">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Rwanda Social Security Board (RSSB)</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Rwanda</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Public PF</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Fund LP / Anchor</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Admaius Capital Partners</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Virunga Africa Fund I</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Private equity / growth / multi-sector</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Pan-Africa</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>2021</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Not separately disclosed (fund size USD 250m)</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>KIFC/RSSB press release / PDF</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>KIFC/RSSB - Virunga Africa Fund I launch (2 Nov 2021)</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>KIFC/RSSB PDF names QIA and RSSB as anchor/cornerstone investors. Fund managed by Admaius, headquartered in Kigali and domiciled in KIFC; targets healthcare, education, digital infrastructure, financial services, and wider economic transformation across Africa.</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>Healthcare; Education; Digital / Technology; Financial Inclusion / Financial Services; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O98"/>
   <conditionalFormatting sqref="N2:N98">
@@ -36614,7 +36735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="16" min="1" max="1"/>
@@ -39511,7 +39632,75 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="45.75" customHeight="1" s="16"/>
+    <row r="43" ht="45.75" customHeight="1" s="16">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Virunga Africa Fund I</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Admaius Capital Partners</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D43" t="n">
+        <v>250</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Private equity / growth / multi-sector</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Pan-Africa</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>1</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>RSSB (Rwanda Social Security Board) - anchor investor (commitment amount not separately disclosed)</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>1</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Qatar Investment Authority (QIA)</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>KIFC/RSSB launch announcement names QIA and RSSB as the two anchor/cornerstone investors in the USD 250m pan-African fund. Managed by Admaius and domiciled in KIFC.</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Healthcare; Education; Digital / Technology; Financial Inclusion / Financial Services; Multi-Sector</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+    </row>
     <row r="44" ht="57" customHeight="1" s="16"/>
     <row r="45" ht="45.75" customHeight="1" s="16"/>
     <row r="46" ht="45.75" customHeight="1" s="16"/>

</xml_diff>

<commit_message>
Add fund vehicles for all 6 new commitments; add QIA to network map
Funds & LP Co-Investors tab — 6 new vehicle rows (44-49):
- South Suez Africa Fund (I, II + Managed Accounts) — GIPF, PE FoF
- Investec Africa PE Fund 2 L.P. — GIPF, pan-Africa PE
- Neoma Africa Fund III (B) L.P. (prev Abraaj) — GIPF, SSA PE
- Actis Africa fund — GIPF, Africa PE
- Growthpoint Investec Africa Properties Ltd — GIPF, Africa RE
- Teranga Capital — FONSIS, Senegal SME impact

network.js: add QIA (Qatar Investment Authority) to DFI_ALIASES so it
renders as a node linked to Virunga Africa Fund I

Regenerate data.js (Funds & LP Co-Investors now 46 rows).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -44421,7 +44421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O43"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="16" min="1" max="1"/>
@@ -47387,9 +47387,417 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="57" customHeight="1" s="16"/>
-    <row r="45" ht="45.75" customHeight="1" s="16"/>
-    <row r="46" ht="45.75" customHeight="1" s="16"/>
+    <row r="44" ht="57" customHeight="1" s="16">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>South Suez Africa Fund (I, II + Managed Accounts)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>South Suez Capital (Pty) Ltd</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Multiple vintages (2006–2015 est.)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>PE Fund of Funds</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Government Institutions Pension Fund (GIPF)</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>GIPF is the only named African PF/SWF LP disclosed. Pan-African PE FoF investing in primaries, secondaries, and co-investments. GIPF FY2023 market value N$2.75bn (~USD 151m). Source: GIPF 2023 Annual Report p.84.</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Multi-Sector (Pan-African PE)</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Fund LP (Fund of Funds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="45.75" customHeight="1" s="16">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Investec Africa Private Equity Fund 2 L.P.</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Investec Asset Management (now Ninety-One)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>c.2013 (est.)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Pan-African (AU member states + Morocco)</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>1</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Government Institutions Pension Fund (GIPF)</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Guernsey-domiciled LP fund. Invests in established African businesses via buyout/growth transactions. Investec AM rebranded to Ninety-One in 2020. Commitment amount undisclosed; GIPF 2023 AR lists fund in unlisted investment programme (p.96).</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="45.75" customHeight="1" s="16">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Neoma Africa Fund III (B) L.P. (previously Abraaj Africa Fund III)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Neoma Capital Partners (formerly Abraaj Group)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>c.2014 (est.; original Abraaj vintage)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Government Institutions Pension Fund (GIPF)</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Cayman Islands LP. Provides growth capital to Sub-Saharan Africa portfolio companies. Originally managed by Abraaj Group; fund transitioned to Neoma Capital Partners after Abraaj bankruptcy 2018. Source: GIPF 2023 AR p.97.</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Generalist</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Actis Africa fund (specific fund not named in AR)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Actis Investment Management Limited</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Africa (Pan-African)</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Government Institutions Pension Fund (GIPF)</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>GIPF 2023 AR lists Actis IM Ltd with 'Africa Private Equity' mandate; specific fund name not stated. FY2023 market value N$101.5m (~USD 5.6m). Source: GIPF 2023 Annual Report p.84.</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Multi-Sector</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Growthpoint Investec Africa Properties Limited</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Growthpoint Properties / Investec</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>c.2016 (est.)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Africa (ex-South Africa): Ghana, Kenya, Morocco, Mozambique, Tanzania, Zambia</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Government Institutions Pension Fund (GIPF)</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Pan-African commercial real estate fund. Primary targets: Ghana, Kenya, Morocco, Mozambique, Tanzania, Zambia. Secondary: Angola, Botswana, Côte d'Ivoire, Cameroon, Ethiopia, Gabon, Mauritius, Namibia, Nigeria, Rwanda, Uganda. Source: GIPF 2023 AR p.96.</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Commercial Real Estate (Pan-African)</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Teranga Capital</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>I&amp;P (Investisseurs &amp; Partenaires) / Local managers</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Private Equity / Impact</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Domestic (Senegal)</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>1</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>FONSIS (Senegal)</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>1</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>European Union / IFAD</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Sonatel; SG Senegal; ASKIA Insurance</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>FONSIS is a founding LP/shareholder alongside I&amp;P (via IPDEV2), Sonatel, SG Senegal, and ASKIA Insurance. EU is a governmental partner providing co-financing. Fund targets Senegalese SMEs via impact investing. Initial raise CFA 3.2bn (~USD 5.5m). Source: Teranga Capital website.</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>SME Finance / Impact</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L46"/>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Deduplicate FONSIS / FONSIS (Senegal) → single FONSIS node
Standardise allocator name to 'FONSIS' in:
- Commitments Database row 109 (Teranga Capital)
- Funds & LP Co-Investors row 49 (Teranga Capital LP field)

Ensures single FONSIS allocator node on network map.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -42737,7 +42737,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>FONSIS (Senegal)</t>
+          <t>FONSIS</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -47761,7 +47761,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>FONSIS (Senegal)</t>
+          <t>FONSIS</t>
         </is>
       </c>
       <c r="I49" t="n">

</xml_diff>

<commit_message>
Add Amethis West Africa commitments: CDC Gabon (H) + CNPS-CI (M)
New Commitments Database rows 110-111:
- CDC Gabon → Amethis West Africa (2014, CIMA zone, Confidence H)
  Named LP in Amethis West Africa fund creation press release alongside
  BOAD and Colina Group (Saham). First PE fund registered in Francophone
  Africa under CIMA Code.
- CNPS-CI (Côte d'Ivoire) → Amethis fund (unspecified, likely AWA)
  Confidence M; disclosed in Pension Policy International / Agence Ecofin
  as investing in "investment funds such as one launched by Amethis".

New Funds tab row 50: Amethis West Africa (€~45m, 2014, CIMA zone)
New Source Library rows 235-236

js/network.js: add BOAD to DFI_ALIASES (Banque Ouest Africaine de
Développement); cache-bust → v=20260608-amethis-boad

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -5784,7 +5784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F234"/>
+  <dimension ref="A1:F236"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="16" min="1" max="2"/>
@@ -13279,6 +13279,70 @@
       <c r="F234" t="inlineStr">
         <is>
           <t>FONSIS confirmed as founding LP/shareholder in Teranga Capital (2016 impact SME fund, Senegal). Added as row 109.</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>CDC Gabon (State pension fund of Gabon)</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Fund manager press release</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Amethis Finance – Announces the Creation of Amethis West Africa (AWA)</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>https://amethis.com/en/amethis-finance-announces-the-creation-of-amethis-west-africa/</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>CDC Gabon confirmed as named LP in Amethis West Africa fund (€40-45m, 2014, CIMA zone). Added as Commitments DB row 110.</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Caisse Nationale de Prévoyance Sociale (CNPS-CI)</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Third-party report</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire's CNPS Assets Grow from $40M to $2B in 13 Years – Pension Policy International (citing Agence Ecofin)</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>https://www.pensionpolicyinternational.com/cote-divoires-cnps-assets-grow-from-40m-to-2b-in-13-years/</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>CNPS-CI reported to invest in "investment funds such as one launched by Amethis and the Africa50 fund". Specific fund name unconfirmed. Added as Commitments DB row 111 with confidence M.</t>
         </is>
       </c>
     </row>
@@ -32885,7 +32949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R109"/>
+  <dimension ref="A1:R111"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="16" min="1" max="1"/>
@@ -42821,6 +42885,188 @@
         </is>
       </c>
       <c r="R109" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>CDC Gabon (State pension fund of Gabon)</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Gabon</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Civil-service PF</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Amethis Finance</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Amethis West Africa</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>CIMA zone (Francophone West &amp; Central Africa)</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>2014</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>Press release</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>Amethis West Africa creation announcement</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>Named LP alongside BOAD (DFI) and Colina Group (Saham) in Amethis West Africa fund creation press release. First PE fund registered in Francophone Africa; structured under CIMA Code for insurance/pension technical reserves.</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>Multi-sector</t>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Caisse Nationale de Prévoyance Sociale (CNPS-CI)</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Public PF</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Amethis Finance</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Amethis fund (unspecified; likely Amethis West Africa)</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>CIMA zone / Francophone Africa</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>c.2014 (est.)</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Reported / Indirect</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>Pension Policy International / Agence Ecofin</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>CNPS-CI reported to have placed assets in "investment funds such as one launched by Amethis and the Africa50 fund" (Agence Ecofin / Pension Policy International). Specific fund name not confirmed; Amethis West Africa most likely given geographic focus on CIMA zone.</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>Multi-sector</t>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr">
         <is>
           <t>Fund LP</t>
         </is>
@@ -44421,7 +44667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="16" min="1" max="1"/>
@@ -47793,6 +48039,75 @@
         </is>
       </c>
       <c r="O49" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Amethis West Africa</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Amethis Finance</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D50" t="n">
+        <v>50</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>CIMA zone (Francophone West &amp; Central Africa)</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>CDC Gabon (State pension fund of Gabon)</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>1</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>BOAD (Banque Ouest Africaine de Développement)</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Colina Group (Saham)</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>First PE fund registered in Francophone Africa; CIMA Code–eligible structure; CNPS-CI (Côte d'Ivoire) also likely LP (M confidence per Pension Policy International).</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Multi-sector</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
         <is>
           <t>Fund LP</t>
         </is>

</xml_diff>

<commit_message>
Dedupe KPLC and CBK allocator nodes: canonicalize Funds tab LP names
Pre-existing duplicate allocator nodes found during preview verification:
- "KPLC Pension Fund" (ARVF I/II Funds tab LP cells) vs canonical
  "Kenya Power & Lighting Co. Pension Fund (KPLC PF)"
- "CBK Pension Fund Kenya (since Oct 2018 second close)" (AfricInvest
  FIVE LP cell) vs canonical "CBK Pension Fund (Kenya, Central Bank of Kenya)"

Both Funds tab cells now use exact canonical allocator names; the CBK
timing detail moved to the co-investor pattern note. Network map now
renders 68 allocator nodes (was 70 with dupes).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -46126,7 +46126,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>KPLC Pension Fund (USD 4m, 2014 — 'first East African pension LP in PE'), NMG Pension Fund (USD 1m, 2015 via STANLIB)</t>
+          <t>Kenya Power &amp; Lighting Co. Pension Fund (KPLC PF) (USD 4m, 2014 — 'first East African pension LP in PE'), NMG Pension Fund (USD 1m, 2015 via STANLIB)</t>
         </is>
       </c>
       <c r="I10" s="2" t="n">
@@ -46201,7 +46201,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>KPLC Pension Fund x2 (likely main + Staff RBS), NMG Pension Fund</t>
+          <t>Kenya Power &amp; Lighting Co. Pension Fund (KPLC PF) x2 (likely main + Staff RBS), NMG Pension Fund</t>
         </is>
       </c>
       <c r="I11" s="2" t="n">
@@ -46639,7 +46639,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>CBK Pension Fund Kenya (since Oct 2018 second close)</t>
+          <t>CBK Pension Fund (Kenya, Central Bank of Kenya)</t>
         </is>
       </c>
       <c r="I17" s="2" t="n">
@@ -46657,7 +46657,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Evergreen platform; CBK Pension Fund Kenya was first African pension LP in 2018; multiple closes since.</t>
+          <t>Evergreen platform; CBK Pension Fund Kenya was first African pension LP in 2018; multiple closes since. CBK Pension Fund LP since Oct 2018 second close.</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">

</xml_diff>

<commit_message>
Reclassify Mergence Lesotho entry as mandate, not fund vehicle
The PODCPF commitment is a managed allocation (~3% of AUM) that Mergence
Lesotho invests via direct unlisted deals — there is no discrete,
publicly named fund vehicle. Changes:

- Commitments DB row 119: commitment type -> "Investment mandate /
  managed account"; deal name -> "Mergence Lesotho unlisted investment
  mandate (PE & infrastructure)"; note explains the classification.
- Funds & LP Co-Investors: removed the pseudo-vehicle row (tab back to
  51 data rows).
- Network map: entry no longer renders as a fund node (mandate-type
  commitments are excluded), consistent with KEPFIC/AOFSA handling.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -43882,7 +43882,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Fund LP / managed account</t>
+          <t>Investment mandate / managed account</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -43892,7 +43892,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Mergence Lesotho unlisted PE &amp; infrastructure portfolio</t>
+          <t>Mergence Lesotho unlisted investment mandate (PE &amp; infrastructure)</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -43937,7 +43937,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>PODCPF (largest Lesotho PF, USD 616m AUM) allocates ~3% to private equity via Mergence Investment Managers Lesotho — the only PE manager in the country. Investments span healthcare, property, agriculture, infrastructure, SMEs incl. medical agriculture project and Maseru office building. Specific fund vehicle name not publicly disclosed.</t>
+          <t>PODCPF (largest Lesotho PF, USD 616m AUM) allocates ~3% to private equity via Mergence Investment Managers Lesotho — the only PE manager in the country. Investments span healthcare, property, agriculture, infrastructure, SMEs incl. medical agriculture project and Maseru office building. Specific fund vehicle name not publicly disclosed. Recorded as a mandate, not a fund vehicle: Mergence manages the allocation via direct unlisted deals; no discrete fund vehicle publicly named.</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
@@ -45551,7 +45551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O55"/>
+  <dimension ref="A1:O54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="16" min="1" max="1"/>
@@ -49268,74 +49268,6 @@
         </is>
       </c>
       <c r="O54" t="inlineStr">
-        <is>
-          <t>Fund LP</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Mergence Lesotho unlisted PE &amp; infrastructure portfolio</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Mergence Investment Managers (Lesotho)</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>2018-ongoing</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Private Equity / Infrastructure</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>Lesotho (80% domestic)</t>
-        </is>
-      </c>
-      <c r="G55" t="n">
-        <v>1</v>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>Public Officers' Defined Contribution Pension Fund (PODCPF)</t>
-        </is>
-      </c>
-      <c r="I55" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>Only PE manager licensed in Lesotho; manages PODCPF ~3% unlisted allocation. Healthcare, agriculture, property, SMEs.</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>Private Equity</t>
-        </is>
-      </c>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>Multi-sector / SME</t>
-        </is>
-      </c>
-      <c r="O55" t="inlineStr">
         <is>
           <t>Fund LP</t>
         </is>

</xml_diff>

<commit_message>
Add DFI LP cross-check updates
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -47920,11 +47920,11 @@
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Norfund, OeEB (Austria)</t>
+          <t>BII; FMO; Norfund; OeEB (Austria)</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -47934,7 +47934,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Historical pioneer fund for East African pension PE participation.</t>
+          <t>Historical pioneer fund for East African pension PE participation. DFI project-database cross-check adds BII and FMO to the existing Norfund/OeEB ARVF I record.</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -48137,11 +48137,11 @@
         </is>
       </c>
       <c r="I13" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>BII (USD 30m), EIB, IFC, Proparco, Swedfund</t>
+          <t>BII (USD 30m); EIB; IFC; Proparco; SIFEM; Swedfund</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -48151,7 +48151,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Single largest East African PE fund with disclosed local-pension cohort.</t>
+          <t>Single largest East African PE fund with disclosed local-pension cohort. DFI project-database cross-check adds SIFEM to the named Catalyst Fund II DFI LP set.</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -48285,11 +48285,11 @@
         </is>
       </c>
       <c r="I15" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>IFC, EIB, BII, Norfund, DEG, Finnfund</t>
+          <t>IFC; EIB; BII; Norfund; DEG; Finnfund; Swedfund</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -48299,7 +48299,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Vantage's 'historical pattern' of substantial SA pension LP base; specific names not publicly itemised.</t>
+          <t>Vantage's 'historical pattern' of substantial SA pension LP base; specific names not publicly itemised. DFI project-database cross-check adds Swedfund to the named Vantage Mezzanine IV DFI LP set.</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -48945,14 +48945,12 @@
           <t>PIC South Africa (historical)</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>multiple</t>
-        </is>
+      <c r="I24" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Various DFIs</t>
+          <t>BII; IFC</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -48962,7 +48960,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>Digital infrastructure; PIC participant.</t>
+          <t>Digital infrastructure; PIC participant. DFI project-database cross-check replaces generic DFI label with named BII and IFC commitments.</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -49874,11 +49872,16 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>FMO</t>
+        </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>NSIA impact report identifies a USD 5m FGF commitment to Verod Growth Fund II.</t>
+          <t>NSIA impact report identifies a USD 5m FGF commitment to Verod Growth Fund II. DFI project-database cross-check identifies FMO as a Verod Capital Growth II investor.</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -49937,11 +49940,16 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>BII; BIO; FMO; IFC; Norfund; Proparco/FISEA</t>
+        </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>NSIA impact report identifies a USD 7.5m FGF commitment to Verod Growth Fund III.</t>
+          <t>NSIA impact report identifies a USD 7.5m FGF commitment to Verod Growth Fund III. DFI project-database cross-check identifies BII, BIO, FMO, IFC, Norfund and Proparco/FISEA as Verod Growth Fund III investors.</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -50205,11 +50213,11 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Dutch Good Growth Fund (DGGF); IFC; EIB</t>
+          <t>Dutch Good Growth Fund (DGGF); IFC; EIB; Norfund; Proparco/FISEA</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -50219,7 +50227,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>VCTF government co-investment helped Oasis domicile the fund locally in Ghana. DGGF TA/legal work helped make the Ghana structure bankable for international DFIs; first close included DGGF, IFC and local investors, with EIB later disclosing an USD 8m commitment.</t>
+          <t>VCTF government co-investment helped Oasis domicile the fund locally in Ghana. DGGF TA/legal work helped make the Ghana structure bankable for international DFIs; first close included DGGF, IFC and local investors, with EIB later disclosing an USD 8m commitment. DFI project-database cross-check adds Norfund and Proparco/FISEA as Oasis Africa Fund LPs.</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -50478,21 +50486,21 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
+          <t>BII; FMO; IFC; IFU</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Cayman Islands LP. Provides growth capital to Sub-Saharan Africa portfolio companies. Originally managed by Abraaj Group; fund transitioned to Neoma Capital Partners after Abraaj bankruptcy 2018. Source: GIPF 2023 AR p.97.</t>
+          <t>Cayman Islands LP. Provides growth capital to Sub-Saharan Africa portfolio companies. Originally managed by Abraaj Group; fund transitioned to Neoma Capital Partners after Abraaj bankruptcy 2018. Source: GIPF 2023 AR p.97. DFI project-database cross-check identifies BII, FMO, IFC and IFU as Neoma/Abraaj Africa Fund III investors.</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -50892,11 +50900,11 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BII; FMO; Finnfund; IFC; IFU; Norfund; Proparco/FISEA; SIFEM; Swedfund</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -50906,7 +50914,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Rare case of multiple named African pension LPs in a USD 900m pan-African PE fund, disclosed via MiDA Advisors / USAID INVEST campaign rather than GP press release.</t>
+          <t>Rare case of multiple named African pension LPs in a USD 900m pan-African PE fund, disclosed via MiDA Advisors / USAID INVEST campaign rather than GP press release. DFI project-database cross-check identifies BII, FMO, Finnfund, IFC, IFU, Norfund, Proparco/FISEA, SIFEM and Swedfund as ADP III LPs/parallel fund investors.</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -51130,11 +51138,11 @@
         </is>
       </c>
       <c r="B4" s="23" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C4" s="23" t="inlineStr">
         <is>
-          <t>Ascent Rift Valley Fund II (ARVF II); Capital Alliance Private Equity I-IV (CAPE); Catalyst Fund II; Growth Investment Partners (GIP) Ghana; Growth Investment Partners (GIP) Zambia; Helios Investors II/III/IV (historical); Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Vantage Mezzanine IV (Pan-African sub-fund); Africa Food Security Fund (AFSF)</t>
+          <t>Growth Investment Partners (GIP) Ghana; Growth Investment Partners (GIP) Zambia; Ascent Rift Valley Fund I (ARVF I); Ascent Rift Valley Fund II (ARVF II); Catalyst Fund II; Helios Investors II/III/IV (historical); Vantage Mezzanine IV (Pan-African sub-fund); Convergence Partners Communications Infrastructure Fund; Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Capital Alliance Private Equity I-IV (CAPE); Africa Food Security Fund (AFSF); Verod Growth Fund III; Neoma Africa Fund III (B) L.P. (previously Abraaj Africa Fund III); African Development Partners III (ADP III)</t>
         </is>
       </c>
       <c r="D4" s="23" t="inlineStr">
@@ -51151,20 +51159,20 @@
     <row r="5" ht="23.25" customHeight="1" s="16">
       <c r="A5" s="23" t="inlineStr">
         <is>
-          <t>AfDB</t>
+          <t>IFC</t>
         </is>
       </c>
       <c r="B5" s="23" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C5" s="23" t="inlineStr">
         <is>
-          <t>AfricInvest FIVE (Financial Inclusion Vehicle); Africa50 (general); Africa50 Infrastructure Acceleration Fund (IAF); Mediterrania Capital II / III / IV; Nigeria Infrastructure Fund (NIF, NSIA sub-fund); Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Africa Food Security Fund (AFSF); InfraCredit</t>
+          <t>Ascent Rift Valley Fund II (ARVF II); Adenia Capital V; Catalyst Fund II; Vantage Mezzanine IV (Pan-African sub-fund); Africa50 Infrastructure Acceleration Fund (IAF); Convergence Partners Communications Infrastructure Fund; Verod Growth Fund III; MedServe oncology and diagnostics expansion; Oasis Africa VC Fund (OAF); Neoma Africa Fund III (B) L.P. (previously Abraaj Africa Fund III); African Development Partners III (ADP III)</t>
         </is>
       </c>
       <c r="D5" s="23" t="inlineStr">
         <is>
-          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
+          <t>World Bank Group investor and disclosure source; active in flagship PE/infrastructure vehicles.</t>
         </is>
       </c>
       <c r="E5" s="23" t="inlineStr">
@@ -51176,20 +51184,20 @@
     <row r="6" ht="34.5" customHeight="1" s="16">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t>Norfund</t>
+          <t>AfDB</t>
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C6" s="23" t="inlineStr">
         <is>
-          <t>Adenia Capital V; AfricInvest FIVE (Financial Inclusion Vehicle); Ascent Rift Valley Fund I (ARVF I); Ascent Rift Valley Fund II (ARVF II); Growth Investment Partners (GIP) Ghana; Vantage Mezzanine IV (Pan-African sub-fund)</t>
+          <t>Mediterrania Capital II / III / IV; AfricInvest FIVE (Financial Inclusion Vehicle); Africa50 (general); Africa50 Infrastructure Acceleration Fund (IAF); Nigeria Infrastructure Fund (NIF, NSIA sub-fund); Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Africa Food Security Fund (AFSF); InfraCredit; Nigeria Infrastructure Debt Fund (NIDF)</t>
         </is>
       </c>
       <c r="D6" s="23" t="inlineStr">
         <is>
-          <t>Frequent DFI co-investor in SME, infrastructure, and financial inclusion vehicles.</t>
+          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
         </is>
       </c>
       <c r="E6" s="23" t="inlineStr">
@@ -51201,40 +51209,40 @@
     <row r="7" ht="34.5" customHeight="1" s="16">
       <c r="A7" s="23" t="inlineStr">
         <is>
-          <t>IFC</t>
+          <t>Norfund</t>
         </is>
       </c>
       <c r="B7" s="23" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Adenia Capital V; Africa50 Infrastructure Acceleration Fund (IAF); Ascent Rift Valley Fund II (ARVF II); Catalyst Fund II; Vantage Mezzanine IV (Pan-African sub-fund); Oasis Africa VC Fund (OAF)</t>
+          <t>Growth Investment Partners (GIP) Ghana; Ascent Rift Valley Fund I (ARVF I); Ascent Rift Valley Fund II (ARVF II); Adenia Capital V; Vantage Mezzanine IV (Pan-African sub-fund); AfricInvest FIVE (Financial Inclusion Vehicle); Verod Growth Fund III; Oasis Africa VC Fund (OAF); African Development Partners III (ADP III)</t>
         </is>
       </c>
       <c r="D7" s="23" t="inlineStr">
         <is>
-          <t>World Bank Group investor and disclosure source; active in flagship PE/infrastructure vehicles.</t>
+          <t>Frequent DFI co-investor in SME, infrastructure, and financial inclusion vehicles.</t>
         </is>
       </c>
       <c r="E7" s="23" t="inlineStr">
         <is>
-          <t>2 (Active)</t>
+          <t>1 (Top tier)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="23.25" customHeight="1" s="16">
       <c r="A8" s="23" t="inlineStr">
         <is>
-          <t>EIB</t>
+          <t>FMO</t>
         </is>
       </c>
       <c r="B8" s="23" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>Adenia Capital V; Catalyst Fund II; Mediterrania Capital II / III / IV; Vantage Mezzanine IV (Pan-African sub-fund); Oasis Africa VC Fund (OAF)</t>
+          <t>Ci-Gaba Fund of Funds; Ascent Rift Valley Fund I (ARVF I); Ascent Rift Valley Fund II (ARVF II); Adenia Capital V; Verod Growth Fund II; Verod Growth Fund III; Neoma Africa Fund III (B) L.P. (previously Abraaj Africa Fund III); African Development Partners III (ADP III)</t>
         </is>
       </c>
       <c r="D8" s="23" t="inlineStr">
@@ -51244,47 +51252,47 @@
       </c>
       <c r="E8" s="23" t="inlineStr">
         <is>
-          <t>2 (Active)</t>
+          <t>1 (Top tier)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="23.25" customHeight="1" s="16">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>FMO</t>
+          <t>Proparco</t>
         </is>
       </c>
       <c r="B9" s="23" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Adenia Capital V; Ascent Rift Valley Fund II (ARVF II); Ci-Gaba Fund of Funds</t>
+          <t>Ascent Rift Valley Fund II (ARVF II); Adenia Capital V; Catalyst Fund II; Verod Growth Fund III; Oasis Africa VC Fund (OAF); African Development Partners III (ADP III)</t>
         </is>
       </c>
       <c r="D9" s="23" t="inlineStr">
         <is>
-          <t>Frequent co-investor across funds and fund-of-funds with African pension/SWF participation.</t>
+          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
         </is>
       </c>
       <c r="E9" s="23" t="inlineStr">
         <is>
-          <t>2 (Active)</t>
+          <t>1 (Top tier)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="23.25" customHeight="1" s="16">
       <c r="A10" s="23" t="inlineStr">
         <is>
-          <t>Proparco</t>
+          <t>EIB</t>
         </is>
       </c>
       <c r="B10" s="23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>Adenia Capital V; Ascent Rift Valley Fund II (ARVF II); Catalyst Fund II</t>
+          <t>Adenia Capital V; Catalyst Fund II; Vantage Mezzanine IV (Pan-African sub-fund); Mediterrania Capital II / III / IV; Oasis Africa VC Fund (OAF)</t>
         </is>
       </c>
       <c r="D10" s="23" t="inlineStr">
@@ -51301,15 +51309,15 @@
     <row r="11" ht="23.25" customHeight="1" s="16">
       <c r="A11" s="23" t="inlineStr">
         <is>
-          <t>DEG</t>
+          <t>IFU</t>
         </is>
       </c>
       <c r="B11" s="23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>Adenia Capital V; Vantage Mezzanine IV (Pan-African sub-fund)</t>
+          <t>AfricInvest FIVE (Financial Inclusion Vehicle); Africa Food Security Fund (AFSF); Neoma Africa Fund III (B) L.P. (previously Abraaj Africa Fund III); African Development Partners III (ADP III)</t>
         </is>
       </c>
       <c r="D11" s="23" t="inlineStr">
@@ -51319,39 +51327,39 @@
       </c>
       <c r="E11" s="23" t="inlineStr">
         <is>
-          <t>3 (Selective / TA)</t>
+          <t>2 (Active)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="23.25" customHeight="1" s="16">
       <c r="A12" s="23" t="inlineStr">
         <is>
-          <t>FSD Africa Investments</t>
+          <t>Swedfund</t>
         </is>
       </c>
       <c r="B12" s="23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>Ci-Gaba Fund of Funds; Rwanda SME Growth Fund</t>
+          <t>Growth Investment Partners (GIP) Zambia; Catalyst Fund II; Vantage Mezzanine IV (Pan-African sub-fund); African Development Partners III (ADP III)</t>
         </is>
       </c>
       <c r="D12" s="23" t="inlineStr">
         <is>
-          <t>Catalytic capital provider focused on local institutional-capital mobilization and product design.</t>
+          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
         </is>
       </c>
       <c r="E12" s="23" t="inlineStr">
         <is>
-          <t>3 (Selective / TA)</t>
+          <t>2 (Active)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="34.5" customHeight="1" s="16">
       <c r="A13" s="23" t="inlineStr">
         <is>
-          <t>KfW</t>
+          <t>DGGF</t>
         </is>
       </c>
       <c r="B13" s="23" t="n">
@@ -51359,7 +51367,7 @@
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>AfricInvest FIVE (Financial Inclusion Vehicle); Oyass Capital; InfraCredit</t>
+          <t>Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Africa Food Security Fund (AFSF); Oasis Africa VC Fund (OAF)</t>
         </is>
       </c>
       <c r="D13" s="23" t="inlineStr">
@@ -51369,47 +51377,47 @@
       </c>
       <c r="E13" s="23" t="inlineStr">
         <is>
-          <t>3 (Selective / TA)</t>
+          <t>2 (Active)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="16">
       <c r="A14" s="23" t="inlineStr">
         <is>
-          <t>MiDA Advisors</t>
+          <t>KfW</t>
         </is>
       </c>
       <c r="B14" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C14" s="23" t="inlineStr">
         <is>
-          <t>AOFSA pooled infrastructure mandates (South Africa); KEPFIC pooled mandates (Kenya)</t>
+          <t>Oyass Capital (SME fund); AfricInvest FIVE (Financial Inclusion Vehicle); InfraCredit</t>
         </is>
       </c>
       <c r="D14" s="23" t="inlineStr">
         <is>
-          <t>Technical-assistance and transaction-advisory provider for pension-consortium infrastructure pipelines.</t>
+          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
         </is>
       </c>
       <c r="E14" s="23" t="inlineStr">
         <is>
-          <t>3 (Selective / TA)</t>
+          <t>2 (Active)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="16">
       <c r="A15" s="23" t="inlineStr">
         <is>
-          <t>Swedfund</t>
+          <t>SIFEM</t>
         </is>
       </c>
       <c r="B15" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>Catalyst Fund II; Growth Investment Partners (GIP) Zambia</t>
+          <t>Adenia Capital V; Catalyst Fund II; African Development Partners III (ADP III)</t>
         </is>
       </c>
       <c r="D15" s="23" t="inlineStr">
@@ -51419,14 +51427,14 @@
       </c>
       <c r="E15" s="23" t="inlineStr">
         <is>
-          <t>3 (Selective / TA)</t>
+          <t>2 (Active)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="23.25" customHeight="1" s="16">
       <c r="A16" s="23" t="inlineStr">
         <is>
-          <t>USAID</t>
+          <t>BIO</t>
         </is>
       </c>
       <c r="B16" s="23" t="n">
@@ -51434,12 +51442,12 @@
       </c>
       <c r="C16" s="23" t="inlineStr">
         <is>
-          <t>AOFSA pooled infrastructure mandates (South Africa); KEPFIC pooled mandates (Kenya)</t>
+          <t>Ascent Rift Valley Fund II (ARVF II); Verod Growth Fund III</t>
         </is>
       </c>
       <c r="D16" s="23" t="inlineStr">
         <is>
-          <t>Technical-assistance provider supporting pension-consortium formation and capacity building.</t>
+          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
         </is>
       </c>
       <c r="E16" s="23" t="inlineStr">
@@ -51451,7 +51459,7 @@
     <row r="17" ht="15" customHeight="1" s="16">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>World Bank / IFC J-CAP</t>
+          <t>DEG</t>
         </is>
       </c>
       <c r="B17" s="23" t="n">
@@ -51459,12 +51467,12 @@
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>AOFSA pooled infrastructure mandates (South Africa); KEPFIC pooled mandates (Kenya)</t>
+          <t>Adenia Capital V; Vantage Mezzanine IV (Pan-African sub-fund)</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>Technical-assistance and market-development provider for pension-consortium structures.</t>
+          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
         </is>
       </c>
       <c r="E17" s="23" t="inlineStr">
@@ -51476,15 +51484,15 @@
     <row r="18" ht="15" customHeight="1" s="16">
       <c r="A18" s="23" t="inlineStr">
         <is>
-          <t>BCEAO</t>
+          <t>European Union / IFAD</t>
         </is>
       </c>
       <c r="B18" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>Africa50 (general)</t>
+          <t>Yield Uganda Investment Fund; Teranga Capital</t>
         </is>
       </c>
       <c r="D18" s="23" t="inlineStr">
@@ -51501,20 +51509,20 @@
     <row r="19" ht="15" customHeight="1" s="16">
       <c r="A19" s="23" t="inlineStr">
         <is>
-          <t>BIO</t>
+          <t>FSD Africa Investments</t>
         </is>
       </c>
       <c r="B19" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" s="23" t="inlineStr">
         <is>
-          <t>Ascent Rift Valley Fund II (ARVF II)</t>
+          <t>Ci-Gaba Fund of Funds; Rwanda SME Growth Fund</t>
         </is>
       </c>
       <c r="D19" s="23" t="inlineStr">
         <is>
-          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
+          <t>Catalytic capital provider focused on local institutional-capital mobilization and product design.</t>
         </is>
       </c>
       <c r="E19" s="23" t="inlineStr">
@@ -51526,15 +51534,15 @@
     <row r="20" ht="15" customHeight="1" s="16">
       <c r="A20" s="23" t="inlineStr">
         <is>
-          <t>Bank Al-Maghrib</t>
+          <t>Finnfund</t>
         </is>
       </c>
       <c r="B20" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C20" s="23" t="inlineStr">
         <is>
-          <t>Africa50 (general)</t>
+          <t>Vantage Mezzanine IV (Pan-African sub-fund); African Development Partners III (ADP III)</t>
         </is>
       </c>
       <c r="D20" s="23" t="inlineStr">
@@ -51551,7 +51559,7 @@
     <row r="21" ht="15" customHeight="1" s="16">
       <c r="A21" s="23" t="inlineStr">
         <is>
-          <t>Batseta Council</t>
+          <t>BOAD</t>
         </is>
       </c>
       <c r="B21" s="23" t="n">
@@ -51559,12 +51567,12 @@
       </c>
       <c r="C21" s="23" t="inlineStr">
         <is>
-          <t>AOFSA pooled infrastructure mandates (South Africa)</t>
+          <t>Amethis West Africa</t>
         </is>
       </c>
       <c r="D21" s="23" t="inlineStr">
         <is>
-          <t>South African retirement-fund industry body supporting AOFSA secretariat/governance.</t>
+          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
         </is>
       </c>
       <c r="E21" s="23" t="inlineStr">
@@ -51576,7 +51584,7 @@
     <row r="22" ht="15" customHeight="1" s="16">
       <c r="A22" s="23" t="inlineStr">
         <is>
-          <t>CDP Group</t>
+          <t>DFC</t>
         </is>
       </c>
       <c r="B22" s="23" t="n">
@@ -51584,7 +51592,7 @@
       </c>
       <c r="C22" s="23" t="inlineStr">
         <is>
-          <t>Mediterrania Capital II / III / IV</t>
+          <t>Adenia Capital V</t>
         </is>
       </c>
       <c r="D22" s="23" t="inlineStr">
@@ -51601,7 +51609,7 @@
     <row r="23" ht="23.25" customHeight="1" s="16">
       <c r="A23" s="23" t="inlineStr">
         <is>
-          <t>CrossBoundary</t>
+          <t>EBID</t>
         </is>
       </c>
       <c r="B23" s="23" t="n">
@@ -51609,12 +51617,12 @@
       </c>
       <c r="C23" s="23" t="inlineStr">
         <is>
-          <t>AOFSA pooled infrastructure mandates (South Africa)</t>
+          <t>Africa Food Security Fund (AFSF)</t>
         </is>
       </c>
       <c r="D23" s="23" t="inlineStr">
         <is>
-          <t>Technical-assistance provider supporting AOFSA pipeline development.</t>
+          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
         </is>
       </c>
       <c r="E23" s="23" t="inlineStr">
@@ -51626,15 +51634,15 @@
     <row r="24" ht="15" customHeight="1" s="16">
       <c r="A24" s="23" t="inlineStr">
         <is>
-          <t>Dutch Good Growth Fund</t>
+          <t>FinDev Canada</t>
         </is>
       </c>
       <c r="B24" s="23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Africa Food Security Fund (AFSF); Oasis Africa VC Fund (OAF)</t>
+          <t>Adenia Capital V</t>
         </is>
       </c>
       <c r="D24" s="23" t="inlineStr">
@@ -51651,7 +51659,7 @@
     <row r="25" ht="15" customHeight="1" s="16">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>FCA Investments</t>
+          <t>GuarantCo / PIDG</t>
         </is>
       </c>
       <c r="B25" s="23" t="n">
@@ -51659,7 +51667,7 @@
       </c>
       <c r="C25" s="23" t="inlineStr">
         <is>
-          <t>Yield Uganda Investment Fund</t>
+          <t>InfraCredit</t>
         </is>
       </c>
       <c r="D25" s="23" t="inlineStr">
@@ -51676,7 +51684,7 @@
     <row r="26" ht="15" customHeight="1" s="16">
       <c r="A26" s="23" t="inlineStr">
         <is>
-          <t>FinDev Canada</t>
+          <t>InfraCo Africa</t>
         </is>
       </c>
       <c r="B26" s="23" t="n">
@@ -51684,7 +51692,7 @@
       </c>
       <c r="C26" s="23" t="inlineStr">
         <is>
-          <t>Adenia Capital V</t>
+          <t>InfraCredit</t>
         </is>
       </c>
       <c r="D26" s="23" t="inlineStr">
@@ -51699,129 +51707,39 @@
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="16">
-      <c r="A27" s="23" t="inlineStr">
-        <is>
-          <t>IFU</t>
-        </is>
-      </c>
-      <c r="B27" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="C27" s="23" t="inlineStr">
-        <is>
-          <t>AfricInvest FIVE (Financial Inclusion Vehicle); Africa Food Security Fund (AFSF)</t>
-        </is>
-      </c>
-      <c r="D27" s="23" t="inlineStr">
-        <is>
-          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
-        </is>
-      </c>
-      <c r="E27" s="23" t="inlineStr">
-        <is>
-          <t>3 (Selective / TA)</t>
-        </is>
-      </c>
+      <c r="A27" s="23" t="n"/>
+      <c r="B27" s="23" t="n"/>
+      <c r="C27" s="23" t="n"/>
+      <c r="D27" s="23" t="n"/>
+      <c r="E27" s="23" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="inlineStr">
-        <is>
-          <t>OeEB</t>
-        </is>
-      </c>
-      <c r="B28" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" s="23" t="inlineStr">
-        <is>
-          <t>Ascent Rift Valley Fund I (ARVF I)</t>
-        </is>
-      </c>
-      <c r="D28" s="23" t="inlineStr">
-        <is>
-          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
-        </is>
-      </c>
-      <c r="E28" s="23" t="inlineStr">
-        <is>
-          <t>3 (Selective / TA)</t>
-        </is>
-      </c>
+      <c r="A28" s="23" t="n"/>
+      <c r="B28" s="23" t="n"/>
+      <c r="C28" s="23" t="n"/>
+      <c r="D28" s="23" t="n"/>
+      <c r="E28" s="23" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="inlineStr">
-        <is>
-          <t>SIFEM</t>
-        </is>
-      </c>
-      <c r="B29" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" s="23" t="inlineStr">
-        <is>
-          <t>Adenia Capital V</t>
-        </is>
-      </c>
-      <c r="D29" s="23" t="inlineStr">
-        <is>
-          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
-        </is>
-      </c>
-      <c r="E29" s="23" t="inlineStr">
-        <is>
-          <t>3 (Selective / TA)</t>
-        </is>
-      </c>
+      <c r="A29" s="23" t="n"/>
+      <c r="B29" s="23" t="n"/>
+      <c r="C29" s="23" t="n"/>
+      <c r="D29" s="23" t="n"/>
+      <c r="E29" s="23" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="16">
-      <c r="A30" s="23" t="inlineStr">
-        <is>
-          <t>Soros Economic Development Fund</t>
-        </is>
-      </c>
-      <c r="B30" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" s="23" t="inlineStr">
-        <is>
-          <t>Yield Uganda Investment Fund</t>
-        </is>
-      </c>
-      <c r="D30" s="23" t="inlineStr">
-        <is>
-          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
-        </is>
-      </c>
-      <c r="E30" s="23" t="inlineStr">
-        <is>
-          <t>3 (Selective / TA)</t>
-        </is>
-      </c>
+      <c r="A30" s="23" t="n"/>
+      <c r="B30" s="23" t="n"/>
+      <c r="C30" s="23" t="n"/>
+      <c r="D30" s="23" t="n"/>
+      <c r="E30" s="23" t="n"/>
     </row>
     <row r="31" ht="109.5" customHeight="1" s="16">
-      <c r="A31" s="23" t="inlineStr">
-        <is>
-          <t>US DFC</t>
-        </is>
-      </c>
-      <c r="B31" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" s="23" t="inlineStr">
-        <is>
-          <t>Adenia Capital V</t>
-        </is>
-      </c>
-      <c r="D31" s="23" t="inlineStr">
-        <is>
-          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
-        </is>
-      </c>
-      <c r="E31" s="23" t="inlineStr">
-        <is>
-          <t>3 (Selective / TA)</t>
-        </is>
-      </c>
+      <c r="A31" s="23" t="n"/>
+      <c r="B31" s="23" t="n"/>
+      <c r="C31" s="23" t="n"/>
+      <c r="D31" s="23" t="n"/>
+      <c r="E31" s="23" t="n"/>
     </row>
     <row r="32" ht="109.5" customHeight="1" s="16"/>
     <row r="33" ht="109.5" customHeight="1" s="16"/>
@@ -51840,106 +51758,10 @@
     <row r="46" ht="23.85" customHeight="1" s="16"/>
     <row r="47" ht="23.85" customHeight="1" s="16"/>
     <row r="48" ht="129.75" customHeight="1" s="16"/>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>EBID</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>1</v>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Africa Food Security Fund (AFSF)</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Co-investor or catalytic-capital provider appearing in retained vehicles with African PF/SWF participation.</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>3 (Selective / TA)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Kuramo Capital Management</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>1</v>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Africa Food Security Fund (AFSF)</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Other named LP / fund-of-funds investor appearing in retained vehicles with African PF/SWF participation.</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>3 (Selective / TA)</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>GuarantCo / PIDG</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>1</v>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>InfraCredit</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Guarantee/catalytic capital provider that established InfraCredit with NSIA via PIDG/GuarantCo.</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>3 (Selective / TA)</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>InfraCo Africa</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>1</v>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>InfraCredit</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>PIDG project-development arm/shareholder capital provider to InfraCredit.</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>3 (Selective / TA)</t>
-        </is>
-      </c>
-    </row>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
   </sheetData>
   <autoFilter ref="A3:E27"/>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Publish high-confidence commitment additions
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -2286,7 +2286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="16" min="1" max="1"/>
@@ -4697,6 +4697,300 @@
       <c r="H65" t="inlineStr">
         <is>
           <t>https://vctf.com.gh/wp-content/uploads/2022/09/Venture-Capital-Annual-report-2015.pdf; https://english.dggf.nl/site/binaries/site-content/collections/documents/2025/11/17/getting-sme-risk-capital-funds-to-first-close/dggf-knowledge-product-getting-sme-risk-capital-funds-to-first-close.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Funds &amp; LP Co-Investors</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>added 2026-06-22</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Enko Impact Credit Fund</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>PIC (mgr for GEPF) (USD 30m)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Named African public pension asset manager commitment to a specific private credit fund, with amount disclosed.</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>https://www.bii.co.uk/en/news-insight/news/bii-and-pic-announce-first-investment-under-new-partnership-to-drive-growth-for-african-businesses/; https://www.ecofinagency.com/news-finances/2411-50773-enko-capital-raises-130mln-for-its-private-credit-fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Funds &amp; LP Co-Investors</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>added 2026-06-22</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Hlayisani Venture Fund II</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>PIC (mgr for GEPF)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Fund manager names PIC as anchor investor in ZAR 500m first close.</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>https://hlayisani.com/news/</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Funds &amp; LP Co-Investors</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>added 2026-06-22</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>African Women Impact Fund (AWIF)</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Motor Industry Retirement Fund (MIRF); Copartes Pension Fund</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>UNECA names African pension funds and amount brought under AWIF initiative; fund-of-funds/gender-lens alternatives vehicle.</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>https://www.uneca.org/stories/african-women-impact-fund-launches-with-usd%2460-million-commitment-to-drive-an-inclusive; https://www.midaadvisors.com/advisory-firm-the-african-women-impact-fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Funds &amp; LP Co-Investors</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>added 2026-06-22</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Kholo Capital Mezzanine Debt Fund I</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Mineworkers Provident Fund; National Fund for Municipal Workers (NFMW)</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>First-close coverage names two South African pension funds as institutional investors in a specific mezzanine/private debt fund.</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>https://www.africaprivateequitynews.com/p/kholo-capital-mezzanine-debt-fund-i-achieves-first-close; https://ffnews.com/newsarticle/debt-fund-kholo-capital-mezzanine-debt-fund-i-achieve-first-close-at-r870m/</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Commitments Database</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>added 2026-06-23</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Africa50 Infrastructure Acceleration Fund (IAF)</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Public Service Superannuation Scheme/Fund Kenya</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Africa50 official release names Public Service Superannuation Fund (Kenya) as a recent IAF commitment; reconciled to existing PSSS institution name.</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>https://www.africa50.com/media/news/article/africa50-infrastructure-acceleration-fund-marks-inaugural-investment-in-port-operator-mass-cereales-al-maghreb/</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Commitments Database</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>added 2026-06-23</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Africa50 Infrastructure Acceleration Fund (IAF)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>CNPS Cameroon</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Africa50 official release names CNPS Cameroon as a recent IAF commitment; distinct from existing AFC equity holding.</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>https://www.africa50.com/media/news/article/africa50-infrastructure-acceleration-fund-marks-inaugural-investment-in-port-operator-mass-cereales-al-maghreb/</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Commitments Database</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>added 2026-06-23</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Africa Credit Opportunities Fund III (ACO Fund 3)</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>GEPF (via PIC)</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>GEPF official annual report names approved allocation to Ninety One Credit Fund / Africa Credit Opportunities Fund III; GP/DFI sources confirm fund first close and co-investor base.</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>https://gepf.co.za/wp-content/uploads/2025/11/GEPF_AR_2025_digital.pdf; https://ninetyone.com/en/newsroom/ninety-one-announces-usd260-million-first-close-of-aco-fund-3; https://www.findevcanada.ca/en/news/findev-canada-commits-usd-20-million-ninety-ones-africa-credit-opportunities-fund-iii-support</t>
         </is>
       </c>
     </row>
@@ -4982,7 +5276,7 @@
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
         <is>
-          <t>Candidate - new 2026 item</t>
+          <t>Added to Commitments Database - 2026-06-22</t>
         </is>
       </c>
       <c r="B4" s="21" t="inlineStr">
@@ -5032,7 +5326,7 @@
       </c>
       <c r="K4" s="21" t="inlineStr">
         <is>
-          <t>Add to Commitments and Fund Vehicles as confirmed first-close/commitments-to-date, with note that final close is pending.</t>
+          <t>Added to Commitments Database, Fund Vehicles, Source Library, Inclusion Audit, and DFI/Other LP patterns where applicable.</t>
         </is>
       </c>
       <c r="L4" s="21" t="inlineStr">
@@ -5614,7 +5908,7 @@
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>Candidate - likely add after amount/source detail check</t>
+          <t>Actioned - added to database 2026-06-23</t>
         </is>
       </c>
       <c r="B12" s="21" t="inlineStr">
@@ -5634,7 +5928,7 @@
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
-          <t>Not yet checked in this sweep.</t>
+          <t>IFC; BII; SIFEM; Standard Bank debt facility; FinDev Canada</t>
         </is>
       </c>
       <c r="F12" s="21" t="inlineStr">
@@ -5654,7 +5948,7 @@
       </c>
       <c r="I12" s="21" t="inlineStr">
         <is>
-          <t>GEPF annual report confirms approved allocation; commitment amount not yet isolated.</t>
+          <t>GEPF annual report confirms approved allocation; Ninety One first close USD 260m; GEPF amount not disclosed.</t>
         </is>
       </c>
       <c r="J12" s="21" t="inlineStr">
@@ -5664,12 +5958,12 @@
       </c>
       <c r="K12" s="21" t="inlineStr">
         <is>
-          <t>Research Ninety One/DFI fund-close disclosures and GEPF note 3.1 for commitment amount; likely add to Commitments Database if allocator-to-fund allocation is sufficiently specific.</t>
+          <t>Added to Commitments Database, Source Library, Inclusion Audit, and fund-level co-investor view.</t>
         </is>
       </c>
       <c r="L12" s="21" t="inlineStr">
         <is>
-          <t>Official GEPF report names a specific African private credit fund allocation approved in FY2024/25.</t>
+          <t>Official GEPF report names a specific African private credit fund allocation approved in FY2024/25; GP/DFI sources confirm ACO Fund 3 first close and co-investor base.</t>
         </is>
       </c>
       <c r="M12" s="21" t="inlineStr">
@@ -5679,7 +5973,7 @@
       </c>
       <c r="N12" s="21" t="inlineStr">
         <is>
-          <t>https://www.pic.gov.za/DocAnnualReports1/PIC%20Integrated%20Annual%20Report%202024.pdf</t>
+          <t>https://ninetyone.com/en/newsroom/ninety-one-announces-usd260-million-first-close-of-aco-fund-3; https://www.findevcanada.ca/en/news/findev-canada-commits-usd-20-million-ninety-ones-africa-credit-opportunities-fund-iii-support</t>
         </is>
       </c>
       <c r="O12" s="21" t="inlineStr">
@@ -5784,7 +6078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G241"/>
+  <dimension ref="A1:G251"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="16" min="1" max="2"/>
@@ -14708,6 +15002,376 @@
       <c r="G241" t="inlineStr">
         <is>
           <t>S240</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>PIC / GEPF</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>DFI / investor press release</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>BII and PIC announce first investment under new partnership to drive growth for African businesses</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>https://www.bii.co.uk/en/news-insight/news/bii-and-pic-announce-first-investment-under-new-partnership-to-drive-growth-for-african-businesses/</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>PIC/GEPF via PIC USD 30m commitment to Enko Impact Credit Fund; BII partnership co-investment evidence.</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>S241</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>PIC / GEPF</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Trade press</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Ecofin Agency ? Enko Capital raises $130mln for its private credit fund</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>https://www.ecofinagency.com/news-finances/2411-50773-enko-capital-raises-130mln-for-its-private-credit-fund</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Enko Impact Credit Fund first close and PIC USD 30m commitment corroboration.</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>S242</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>PIC / GEPF</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Fund manager press release</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Hlayisani Capital ? Hlayisani Venture Fund II first close / anchored by PIC and SA SME Fund</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>https://hlayisani.com/news/</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Hlayisani Venture Fund II ZAR 500m first close anchored by PIC and SA SME Fund.</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>S243</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>MIRF / Copartes Pension Fund</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>UN agency press release</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>UNECA ? African Women Impact Fund launches with USD 60 million commitment</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>https://www.uneca.org/stories/african-women-impact-fund-launches-with-usd%2460-million-commitment-to-drive-an-inclusive</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>MIRF and Copartes Pension Fund brought USD 45m under AWIF as part of USD 60m first commitment with BADEA.</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>S244</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>MIRF / Copartes Pension Fund</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Advisor case study</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>MiDA Advisors ? The African Women Impact Fund</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>https://www.midaadvisors.com/advisory-firm-the-african-women-impact-fund</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>AWIF structure, investor mobilization context, and African pension capital participation.</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>S245</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Mineworkers Provident Fund / NFMW</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Trade press</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Africa Private Equity News ? Kholo Capital Mezzanine Debt Fund I achieves first close</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>https://www.africaprivateequitynews.com/p/kholo-capital-mezzanine-debt-fund-i-achieves-first-close</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Kholo Capital Mezzanine Debt Fund I R870m first close and named South African pension LPs.</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>S246</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Mineworkers Provident Fund / NFMW</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Trade press</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Fintech Finance ? Debt fund Kholo Capital Mezzanine Debt Fund I achieve first close at R870m</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>https://ffnews.com/newsarticle/debt-fund-kholo-capital-mezzanine-debt-fund-i-achieve-first-close-at-r870m/</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Corroborates Kholo Capital Mezzanine Debt Fund I first close and institutional investor participation.</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>S247</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Africa50 IAF / Kenya PSSS / CNPS Cameroon</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Press release</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Africa50 Infrastructure Acceleration Fund marks inaugural investment in port operator Mass Cereales al Maghreb</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>https://www.africa50.com/media/news/article/africa50-infrastructure-acceleration-fund-marks-inaugural-investment-in-port-operator-mass-cereales-al-maghreb/</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Africa50 IAF recent commitments from DBSA, Axian Group, Public Service Superannuation Fund (Kenya), and CNPS Cameroon.</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>S248</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Ninety One</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Fund manager press release</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Ninety One announces USD 260 million first close of ACO Fund 3</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>https://ninetyone.com/en/newsroom/ninety-one-announces-usd260-million-first-close-of-aco-fund-3</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>ACO Fund 3 first close, fund strategy, anchor LPs IFC, BII, SIFEM, and Standard Bank debt facility.</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>S249</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>FinDev Canada / Ninety One</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>DFI press release</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>FinDev Canada commits USD 20 million to Ninety One Africa Credit Opportunities Fund III</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>https://www.findevcanada.ca/en/news/findev-canada-commits-usd-20-million-ninety-ones-africa-credit-opportunities-fund-iii-support</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Additional DFI co-investor evidence for Ninety One Africa Credit Opportunities Fund III.</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>S250</t>
         </is>
       </c>
     </row>
@@ -34314,7 +34978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S119"/>
+  <dimension ref="A1:S128"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="16" min="1" max="1"/>
@@ -45743,6 +46407,873 @@
       <c r="S119" t="inlineStr">
         <is>
           <t>S239;S240</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>PIC (mgr for GEPF)</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Public PF asset manager</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Fund LP / co-investor</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Enko Capital</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Enko Impact Credit Fund</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Private credit</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="J120" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>Press release / trade press</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>BII / PIC partnership announcement; Ecofin Enko first-close coverage</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>PIC committed USD 30m to Enko Impact Credit Fund as the first investment under the BII-PIC partnership. BII committed USD 25m; Ecofin reports a USD 130m first close and names PIC among key investors. Fund provides private credit to mid-sized businesses in Sub-Saharan Africa.</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>SME / Mid-market finance</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="S120" t="inlineStr">
+        <is>
+          <t>S241;S242</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>PIC (mgr for GEPF)</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Public PF asset manager</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Fund LP / anchor investor</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Hlayisani Capital</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Hlayisani Venture Fund II</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>VC / growth equity</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Share of ZAR 500m first close</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>ZAR</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>Fund manager press release</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>Hlayisani Venture Fund II first-close announcement</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>Hlayisani states that Hlayisani Venture Fund II achieved a ZAR 500m first close anchored by PIC and SA SME Fund. Fund backs high-growth South African businesses, including technology-enabled SMEs and platforms.</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>Technology-enabled SMEs</t>
+        </is>
+      </c>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="S121" t="inlineStr">
+        <is>
+          <t>S243</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Motor Industry Retirement Fund (MIRF)</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Multi-employer PF</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Fund-of-funds allocation / initiative anchor</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>African Women Impact Fund / RisCura</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>African Women Impact Fund (AWIF)</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Fund of Funds / gender-lens private markets</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Share of USD 45m MIRF/Copartes allocation</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>UN agency press release / advisor case study</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>UNECA AWIF launch; MiDA AWIF case study</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>UNECA reports MIRF and Copartes Pension Fund brought USD 45m of assets under the African Women Impact Fund initiative, alongside a USD 15m BADEA commitment for a USD 60m first commitment. AWIF is a fund-of-funds/gender-lens platform investing in women fund managers and gender-diverse teams.</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>Fund of Funds</t>
+        </is>
+      </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>Gender-lens / women fund managers</t>
+        </is>
+      </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>Fund of Funds LP</t>
+        </is>
+      </c>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>S244;S245</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Copartes Pension Fund</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Pension fund</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Fund-of-funds allocation / initiative anchor</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>African Women Impact Fund / RisCura</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>African Women Impact Fund (AWIF)</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Fund of Funds / gender-lens private markets</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Share of USD 45m MIRF/Copartes allocation</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>UN agency press release / advisor case study</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>UNECA AWIF launch; MiDA AWIF case study</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>UNECA reports MIRF and Copartes Pension Fund brought USD 45m of assets under the African Women Impact Fund initiative, alongside a USD 15m BADEA commitment for a USD 60m first commitment. Individual split between MIRF and Copartes was not disclosed publicly.</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>Fund of Funds</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>Gender-lens / women fund managers</t>
+        </is>
+      </c>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>Fund of Funds LP</t>
+        </is>
+      </c>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>S244;S245</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Mineworkers Provident Fund</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Multi-employer PF</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Kholo Capital</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Kholo Capital Mezzanine Debt Fund I</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Private credit / mezzanine debt</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Southern Africa</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Share of ZAR 870m first close</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>ZAR</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>Trade press</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>Kholo Capital Mezzanine Debt Fund I first-close coverage</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>Kholo Capital Mezzanine Debt Fund I reached a ZAR 870m first close with institutional investors including Mineworkers Provident Fund and National Fund for Municipal Workers. The fund provides mezzanine/private debt to mid-market businesses in Southern Africa.</t>
+        </is>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>Mid-market finance</t>
+        </is>
+      </c>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="S124" t="inlineStr">
+        <is>
+          <t>S246;S247</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>National Fund for Municipal Workers (NFMW)</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Multi-employer PF</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Kholo Capital</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Kholo Capital Mezzanine Debt Fund I</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Private credit / mezzanine debt</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Southern Africa</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Share of ZAR 870m first close</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>ZAR</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>Trade press</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>Kholo Capital Mezzanine Debt Fund I first-close coverage</t>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>Kholo Capital Mezzanine Debt Fund I reached a ZAR 870m first close with institutional investors including Mineworkers Provident Fund and National Fund for Municipal Workers. Later coverage reported final close at about ZAR 1.4bn, but allocator-level final-close amounts were not publicly split.</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>Mid-market finance</t>
+        </is>
+      </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>S246;S247</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Public Service Superannuation Scheme (PSSS)</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Public PF</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Africa50</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Africa50 Infrastructure Acceleration Fund (IAF)</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Pan-Africa</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>2025</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>Press release</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>Africa50 MCM inaugural investment announcement May 2025</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>Africa50 stated that IAF's inaugural MCM transaction followed recent commitments from DBSA, Axian Group, Public Service Superannuation Fund (Kenya), and CNPS Cameroon, adding to first-close capital. Name reconciled to existing dashboard institution Public Service Superannuation Scheme (PSSS).</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>S248</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>CNPS Cameroon</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Cameroon</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Public PF</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Africa50</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Africa50 Infrastructure Acceleration Fund (IAF)</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Pan-Africa</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>2025</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>Press release</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>Africa50 MCM inaugural investment announcement May 2025</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>Africa50 stated that IAF's inaugural MCM transaction followed recent commitments from DBSA, Axian Group, Public Service Superannuation Fund (Kenya), and CNPS Cameroon, adding to first-close capital. Distinct from CNPS Cameroon's existing AFC equity-shareholder row.</t>
+        </is>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>Real Assets / Infrastructure Equity</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>S248</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>GEPF (via PIC)</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Public PF (via mgr)</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Ninety One</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Africa Credit Opportunities Fund III (ACO Fund 3)</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Private credit</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Africa + emerging markets</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>2024/25</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>Annual report / GP press release</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>GEPF annual report; Ninety One ACO Fund 3 first close</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>GEPF 2025 annual report names an approved allocation to the Ninety One Credit Fund / Africa Credit Opportunities Fund III inside the Pan-African private markets portfolio. Ninety One reported ACO Fund 3 first close at USD 260m with IFC, BII and SIFEM as anchor LPs plus a Standard Bank debt facility; FinDev Canada later committed USD 20m.</t>
+        </is>
+      </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>SME / Mid-market finance; Infrastructure</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>S219;S249;S250</t>
         </is>
       </c>
     </row>
@@ -47341,7 +48872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O54"/>
+  <dimension ref="A1:O59"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="16" min="1" max="1"/>
@@ -48699,7 +50230,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>222.5 first close (&gt;275 mobilised)</t>
+          <t>222.5 first close (&gt;275 mobilised; later commitments added in 2025)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -48714,30 +50245,30 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>5+ named</t>
+          <t>7+ named</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>NSIA Nigeria, CDC Sénégal, CDC Benin, CNSS Togo, CDG Invest Morocco</t>
+          <t>NSIA Nigeria, CDC Senegal, CDC Benin, CNSS Togo, CDG Invest Morocco, Public Service Superannuation Scheme/Fund Kenya, CNPS Cameroon</t>
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>AfDB, IFC</t>
+          <t>AfDB, IFC, DBSA</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Attijariwafa Bank (Morocco), Arab Bank for Economic Development in Africa, West African Development Bank (BOAD)</t>
+          <t>Attijariwafa Bank (Morocco), Arab Bank for Economic Development in Africa, West African Development Bank (BOAD), Axian Group</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>First major pan-African infra fund MAJORITY-funded by African institutions. Africa50's flagship LP-style vehicle.</t>
+          <t>First major pan-African infra fund majority-funded by African institutions. May 2025 Africa50 release adds Kenya PSSS/PSSF and CNPS Cameroon as recent African PF LPs.</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -51066,6 +52597,352 @@
         </is>
       </c>
       <c r="O54" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Enko Impact Credit Fund</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Enko Capital</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>130</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Private credit</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>PIC (mgr for GEPF) (USD 30m)</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>1</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>BII (USD 25m)</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>SICOM Global Fund; other unnamed African pension funds and institutional investors</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>BII-PIC partnership first investment; Ecofin reports USD 130m first close, with PIC USD 30m and BII USD 25m commitments.</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>SME / Mid-market finance</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Hlayisani Venture Fund II</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Hlayisani Capital</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>~27 (ZAR 500m first close)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>VC / growth equity</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>1</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>PIC (mgr for GEPF)</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>SA SME Fund</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>ZAR 500m first close anchored by PIC and SA SME Fund; South African venture/growth fund for technology-enabled SMEs and platforms.</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Technology-enabled SMEs</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>African Women Impact Fund (AWIF)</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>African Women Impact Fund / RisCura</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>60</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Fund of Funds / gender-lens private markets</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>2</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Motor Industry Retirement Fund (MIRF); Copartes Pension Fund (combined USD 45m under AWIF initiative)</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>1</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>BADEA (USD 15m)</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>USD 60m first commitment combines USD 45m from MIRF/Copartes with USD 15m BADEA; AWIF backs women fund managers and gender-diverse investment teams.</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Fund of Funds</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Gender-lens / women fund managers</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>Fund of Funds LP</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Kholo Capital Mezzanine Debt Fund I</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Kholo Capital</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>~47 at first close (ZAR 870m); later ZAR 1.4bn final close</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Private credit / mezzanine debt</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Southern Africa</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>2</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Mineworkers Provident Fund; National Fund for Municipal Workers (NFMW)</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Other institutional investors not individually split in public first-close coverage</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>First close named two South African pension funds; fund provides mezzanine/private debt to mid-market businesses in Southern Africa.</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>Mid-market finance</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>Fund LP</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Africa Credit Opportunities Fund III (ACO Fund 3)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Ninety One</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2024/25</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>260 first close</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Private credit</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Africa + emerging markets</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>GEPF (via PIC) (amount not disclosed)</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>4</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>IFC, BII, SIFEM, FinDev Canada</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Standard Bank USD 45m debt facility</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>GEPF-approved allocation to specific Ninety One African credit fund; GP first-close source names DFI anchors and Standard Bank facility.</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>SME / Mid-market finance; Infrastructure</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
         <is>
           <t>Fund LP</t>
         </is>
@@ -51087,7 +52964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="16" min="1" max="1"/>
@@ -51138,11 +53015,11 @@
         </is>
       </c>
       <c r="B4" s="23" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C4" s="23" t="inlineStr">
         <is>
-          <t>Growth Investment Partners (GIP) Ghana; Growth Investment Partners (GIP) Zambia; Ascent Rift Valley Fund I (ARVF I); Ascent Rift Valley Fund II (ARVF II); Catalyst Fund II; Helios Investors II/III/IV (historical); Vantage Mezzanine IV (Pan-African sub-fund); Convergence Partners Communications Infrastructure Fund; Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Capital Alliance Private Equity I-IV (CAPE); Africa Food Security Fund (AFSF); Verod Growth Fund III; Neoma Africa Fund III (B) L.P. (previously Abraaj Africa Fund III); African Development Partners III (ADP III)</t>
+          <t>Growth Investment Partners (GIP) Ghana; Growth Investment Partners (GIP) Zambia; Ascent Rift Valley Fund I (ARVF I); Ascent Rift Valley Fund II (ARVF II); Catalyst Fund II; Helios Investors II/III/IV (historical); Vantage Mezzanine IV (Pan-African sub-fund); Convergence Partners Communications Infrastructure Fund; Sahel Capital Fund for Agricultural Finance in Nigeria (FAFIN); Capital Alliance Private Equity I-IV (CAPE); Africa Food Security Fund (AFSF); Verod Growth Fund III; Neoma Africa Fund III (B) L.P. (previously Abraaj Africa Fund III); African Development Partners III (ADP III); Enko Impact Credit Fund</t>
         </is>
       </c>
       <c r="D4" s="23" t="inlineStr">
@@ -51758,10 +53635,31 @@
     <row r="46" ht="23.85" customHeight="1" s="16"/>
     <row r="47" ht="23.85" customHeight="1" s="16"/>
     <row r="48" ht="129.75" customHeight="1" s="16"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>BADEA</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>African Women Impact Fund (AWIF)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Catalytic commitment alongside African pension capital in gender-lens fund-of-funds platform.</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>3 (Selective / TA)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:E27"/>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Fix broken source links and add link audit
</commit_message>
<xml_diff>
--- a/african_pf and swf_dataset_5.13.26.xlsx
+++ b/african_pf and swf_dataset_5.13.26.xlsx
@@ -2220,6 +2220,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="15" customHeight="1" s="16">
       <c r="A19" s="18" t="inlineStr">
         <is>
@@ -2235,6 +2236,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>
@@ -2521,7 +2523,7 @@
       </c>
       <c r="H6" s="23" t="inlineStr">
         <is>
-          <t>https://archive.fsdafrica.org/arm-harith-and-fsd-africa-investments-announce-gbp-10m-commitment-to-unlock-nigerian-pension-funds-and-catalyse-local-capital-for-infrastructure/</t>
+          <t>https://fsdafrica.org/nairobi-15-april-2025-10am-eat-fsd-africa-investments-fsdai-the-uk-backed-specialist-development-finance-investor-is-investing-gbp-10-million-into-arm-hariths-climate-and-transition-in/</t>
         </is>
       </c>
     </row>
@@ -7877,7 +7879,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>PSSSF investment guidelines / Annual report</t>
+          <t>PSSSF official website</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -7887,7 +7889,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>https://www.psssf.go.tz/uploads/publication/37Publication2023-05-022267.pdf</t>
+          <t>https://www.psssf.go.tz/</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -9098,7 +9100,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Savannah Impact Advisory (Manager of Ci Gaba FoF)</t>
+          <t>Savannah Impact Advisory - Ci-Gaba Fund page</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -9108,7 +9110,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>https://siaghana.com/our-about/</t>
+          <t>https://www.siaghana.com/ci-gaba-fund</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -9505,7 +9507,7 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>AVCA — AfricInvest FIVE second close brings Norfund, IFU, CBK Pension Fund as investors (Oct 2018)</t>
+          <t>AfricInvest - FIVE second close brings Norfund, IFU, CBK Pension Fund as investors (Oct 2018)</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -9515,7 +9517,7 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>https://www.avca-africa.org/newsroom/member-news/2018/africinvest-s-five-achieves-its-second-close-bringing-norfund-ifu-and-cbk-pension-fund-as-investors/</t>
+          <t>https://www.africinvest.com/news-and-media/news/africinvest-s-five-achieves-its-second-close-bringing-norfund-ifu-and-cbk-pension-fund-as-investors/</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -9579,7 +9581,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>AVCA — AfricInvest FIVE fourth close (2019)</t>
+          <t>AfricInvest - FIVE fourth close brings AfDB as investor (2019)</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -9589,7 +9591,7 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>https://www.avca-africa.org/newsroom/member-news/2019/africinvest-s-five-achieves-fourth-close/</t>
+          <t>https://www.africinvest.com/news-and-media/news/africinvest-s-permanent-vehicle-five-achieves-its-fourth-close-bringing-afdb-as-investor/</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -12095,7 +12097,7 @@
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>Prosper Africa — U.S., Kenyan and South African Pension Funds Commit Over $94m to African PE &amp; Infrastructure</t>
+          <t>Africa PSA mirror - U.S., Kenyan and South African Pension Funds Commit Over $94m to African PE &amp; Infrastructure</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
@@ -12105,7 +12107,7 @@
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>https://www.prosperafrica.gov/news/impact-story/u-s-kenyan-and-south-african-pension-funds-commit-over-94-million-to-african-private-equity-infrastructure/</t>
+          <t>https://www.africapsa.org/news/u-s-kenyan-and-south-african-pension-funds-commit-over-94-million-to-african-private-equity-infrastructure/</t>
         </is>
       </c>
       <c r="F163" s="2" t="inlineStr">
@@ -15407,6 +15409,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="16">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -15830,6 +15833,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="23.25" customHeight="1" s="16">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -16704,6 +16708,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="16">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -16711,6 +16716,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="23.25" customHeight="1" s="16">
       <c r="A5" s="1" t="inlineStr">
         <is>
@@ -16819,6 +16825,8 @@
         <v>0.19</v>
       </c>
     </row>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="16">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -17092,6 +17100,8 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
+    <row r="31"/>
     <row r="32" ht="15" customHeight="1" s="16">
       <c r="A32" s="8" t="inlineStr">
         <is>
@@ -28714,6 +28724,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="23.25" customHeight="1" s="16">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -47495,7 +47506,7 @@
       </c>
       <c r="P2" s="26" t="inlineStr">
         <is>
-          <t>https://archive.fsdafrica.org/arm-harith-and-fsd-africa-investments-announce-gbp-10m-commitment-to-unlock-nigerian-pension-funds-and-catalyse-local-capital-for-infrastructure/</t>
+          <t>https://fsdafrica.org/nairobi-15-april-2025-10am-eat-fsd-africa-investments-fsdai-the-uk-backed-specialist-development-finance-investor-is-investing-gbp-10-million-into-arm-hariths-climate-and-transition-in/</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -48896,6 +48907,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="45.75" customHeight="1" s="16">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -52981,6 +52993,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="45.75" customHeight="1" s="16">
       <c r="A3" s="24" t="inlineStr">
         <is>
@@ -53707,6 +53720,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="23.25" customHeight="1" s="16">
       <c r="A3" s="1" t="inlineStr">
         <is>

</xml_diff>